<commit_message>
first test Russian case
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA81445-66AA-4436-8BF0-DFE7A6BE6924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF8D40CF-9715-4467-9C20-76336593EF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="83">
   <si>
     <t>Commodities</t>
   </si>
@@ -10086,7 +10086,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68B577B-1347-43AB-A697-F4519763B965}">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -10760,6 +10760,666 @@
         <v>0</v>
       </c>
     </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62" t="s">
+        <v>15</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>12</v>
+      </c>
+      <c r="B63" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>12</v>
+      </c>
+      <c r="B64" t="s">
+        <v>19</v>
+      </c>
+      <c r="C64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>12</v>
+      </c>
+      <c r="B65" t="s">
+        <v>21</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>12</v>
+      </c>
+      <c r="B66" t="s">
+        <v>23</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>12</v>
+      </c>
+      <c r="B67" t="s">
+        <v>25</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>12</v>
+      </c>
+      <c r="B68" t="s">
+        <v>27</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>12</v>
+      </c>
+      <c r="B69" t="s">
+        <v>29</v>
+      </c>
+      <c r="C69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>12</v>
+      </c>
+      <c r="B70" t="s">
+        <v>31</v>
+      </c>
+      <c r="C70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>12</v>
+      </c>
+      <c r="B71" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>12</v>
+      </c>
+      <c r="B72" t="s">
+        <v>35</v>
+      </c>
+      <c r="C72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>12</v>
+      </c>
+      <c r="B73" t="s">
+        <v>37</v>
+      </c>
+      <c r="C73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>12</v>
+      </c>
+      <c r="B74" t="s">
+        <v>39</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>12</v>
+      </c>
+      <c r="B75" t="s">
+        <v>41</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>12</v>
+      </c>
+      <c r="B76" t="s">
+        <v>43</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>12</v>
+      </c>
+      <c r="B77" t="s">
+        <v>45</v>
+      </c>
+      <c r="C77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>12</v>
+      </c>
+      <c r="B78" t="s">
+        <v>46</v>
+      </c>
+      <c r="C78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>12</v>
+      </c>
+      <c r="B79" t="s">
+        <v>48</v>
+      </c>
+      <c r="C79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>12</v>
+      </c>
+      <c r="B80" t="s">
+        <v>49</v>
+      </c>
+      <c r="C80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>12</v>
+      </c>
+      <c r="B81" t="s">
+        <v>51</v>
+      </c>
+      <c r="C81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>12</v>
+      </c>
+      <c r="B82" t="s">
+        <v>52</v>
+      </c>
+      <c r="C82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>12</v>
+      </c>
+      <c r="B83" t="s">
+        <v>54</v>
+      </c>
+      <c r="C83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>12</v>
+      </c>
+      <c r="B84" t="s">
+        <v>56</v>
+      </c>
+      <c r="C84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>12</v>
+      </c>
+      <c r="B85" t="s">
+        <v>58</v>
+      </c>
+      <c r="C85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>12</v>
+      </c>
+      <c r="B86" t="s">
+        <v>59</v>
+      </c>
+      <c r="C86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>12</v>
+      </c>
+      <c r="B87" t="s">
+        <v>38</v>
+      </c>
+      <c r="C87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>12</v>
+      </c>
+      <c r="B88" t="s">
+        <v>16</v>
+      </c>
+      <c r="C88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>12</v>
+      </c>
+      <c r="B89" t="s">
+        <v>28</v>
+      </c>
+      <c r="C89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>12</v>
+      </c>
+      <c r="B90" t="s">
+        <v>44</v>
+      </c>
+      <c r="C90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>12</v>
+      </c>
+      <c r="B91" t="s">
+        <v>62</v>
+      </c>
+      <c r="C91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>12</v>
+      </c>
+      <c r="B92" t="s">
+        <v>22</v>
+      </c>
+      <c r="C92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>12</v>
+      </c>
+      <c r="B93" t="s">
+        <v>63</v>
+      </c>
+      <c r="C93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>12</v>
+      </c>
+      <c r="B94" t="s">
+        <v>66</v>
+      </c>
+      <c r="C94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>12</v>
+      </c>
+      <c r="B95" t="s">
+        <v>24</v>
+      </c>
+      <c r="C95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>12</v>
+      </c>
+      <c r="B96" t="s">
+        <v>18</v>
+      </c>
+      <c r="C96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>12</v>
+      </c>
+      <c r="B97" t="s">
+        <v>42</v>
+      </c>
+      <c r="C97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>12</v>
+      </c>
+      <c r="B98" t="s">
+        <v>30</v>
+      </c>
+      <c r="C98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>12</v>
+      </c>
+      <c r="B99" t="s">
+        <v>64</v>
+      </c>
+      <c r="C99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>12</v>
+      </c>
+      <c r="B100" t="s">
+        <v>67</v>
+      </c>
+      <c r="C100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>12</v>
+      </c>
+      <c r="B101" t="s">
+        <v>68</v>
+      </c>
+      <c r="C101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>12</v>
+      </c>
+      <c r="B102" t="s">
+        <v>70</v>
+      </c>
+      <c r="C102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>12</v>
+      </c>
+      <c r="B103" t="s">
+        <v>71</v>
+      </c>
+      <c r="C103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>12</v>
+      </c>
+      <c r="B104" t="s">
+        <v>20</v>
+      </c>
+      <c r="C104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>12</v>
+      </c>
+      <c r="B105" t="s">
+        <v>53</v>
+      </c>
+      <c r="C105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>12</v>
+      </c>
+      <c r="B106" t="s">
+        <v>26</v>
+      </c>
+      <c r="C106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>12</v>
+      </c>
+      <c r="B107" t="s">
+        <v>75</v>
+      </c>
+      <c r="C107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>12</v>
+      </c>
+      <c r="B108" t="s">
+        <v>34</v>
+      </c>
+      <c r="C108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>12</v>
+      </c>
+      <c r="B109" t="s">
+        <v>32</v>
+      </c>
+      <c r="C109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>12</v>
+      </c>
+      <c r="B110" t="s">
+        <v>60</v>
+      </c>
+      <c r="C110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>12</v>
+      </c>
+      <c r="B111" t="s">
+        <v>74</v>
+      </c>
+      <c r="C111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>12</v>
+      </c>
+      <c r="B112" t="s">
+        <v>55</v>
+      </c>
+      <c r="C112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>12</v>
+      </c>
+      <c r="B113" t="s">
+        <v>77</v>
+      </c>
+      <c r="C113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>12</v>
+      </c>
+      <c r="B114" t="s">
+        <v>36</v>
+      </c>
+      <c r="C114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>12</v>
+      </c>
+      <c r="B115" t="s">
+        <v>50</v>
+      </c>
+      <c r="C115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>12</v>
+      </c>
+      <c r="B116" t="s">
+        <v>40</v>
+      </c>
+      <c r="C116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>12</v>
+      </c>
+      <c r="B117" t="s">
+        <v>57</v>
+      </c>
+      <c r="C117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>12</v>
+      </c>
+      <c r="B118" t="s">
+        <v>47</v>
+      </c>
+      <c r="C118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>12</v>
+      </c>
+      <c r="B119" t="s">
+        <v>78</v>
+      </c>
+      <c r="C119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>12</v>
+      </c>
+      <c r="B120" t="s">
+        <v>79</v>
+      </c>
+      <c r="C120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>12</v>
+      </c>
+      <c r="B121" t="s">
+        <v>81</v>
+      </c>
+      <c r="C121">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
run dummy data for Russian case
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2C3AFA-9616-498F-8081-1155D6067C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD0EFF4-3304-4C53-8C27-D82BD6D5F307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1415" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="81">
   <si>
     <t>Commodities</t>
   </si>
@@ -975,7 +975,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B140"/>
+  <dimension ref="A1:B139"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2084,17 +2084,9 @@
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B139" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A140" t="s">
-        <v>77</v>
-      </c>
-      <c r="B140" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2105,7 +2097,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I273"/>
+  <dimension ref="A1:I277"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -10022,6 +10014,122 @@
         <v>0</v>
       </c>
       <c r="I273">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A274" t="s">
+        <v>11</v>
+      </c>
+      <c r="B274" t="s">
+        <v>77</v>
+      </c>
+      <c r="C274" t="s">
+        <v>20</v>
+      </c>
+      <c r="D274">
+        <v>500</v>
+      </c>
+      <c r="E274">
+        <v>500</v>
+      </c>
+      <c r="F274">
+        <v>1</v>
+      </c>
+      <c r="G274">
+        <v>5</v>
+      </c>
+      <c r="H274">
+        <v>0</v>
+      </c>
+      <c r="I274">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="275" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A275" t="s">
+        <v>12</v>
+      </c>
+      <c r="B275" t="s">
+        <v>77</v>
+      </c>
+      <c r="C275" t="s">
+        <v>20</v>
+      </c>
+      <c r="D275">
+        <v>500</v>
+      </c>
+      <c r="E275">
+        <v>500</v>
+      </c>
+      <c r="F275">
+        <v>1</v>
+      </c>
+      <c r="G275">
+        <v>5</v>
+      </c>
+      <c r="H275">
+        <v>0</v>
+      </c>
+      <c r="I275">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="276" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A276" t="s">
+        <v>12</v>
+      </c>
+      <c r="B276" t="s">
+        <v>15</v>
+      </c>
+      <c r="C276" t="s">
+        <v>16</v>
+      </c>
+      <c r="D276">
+        <v>500</v>
+      </c>
+      <c r="E276">
+        <v>500</v>
+      </c>
+      <c r="F276">
+        <v>10000</v>
+      </c>
+      <c r="G276">
+        <v>5</v>
+      </c>
+      <c r="H276">
+        <v>0</v>
+      </c>
+      <c r="I276">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="277" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A277" t="s">
+        <v>12</v>
+      </c>
+      <c r="B277" t="s">
+        <v>17</v>
+      </c>
+      <c r="C277" t="s">
+        <v>18</v>
+      </c>
+      <c r="D277">
+        <v>500</v>
+      </c>
+      <c r="E277">
+        <v>500</v>
+      </c>
+      <c r="F277">
+        <v>10000</v>
+      </c>
+      <c r="G277">
+        <v>5</v>
+      </c>
+      <c r="H277">
+        <v>0</v>
+      </c>
+      <c r="I277">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
remove duplicate FI connections
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAE517D-064C-4547-8345-FC6B9ABED5F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FE2CB3-5DD6-49BE-895E-56F8D0BC7B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1424" uniqueCount="82">
   <si>
     <t>Commodities</t>
   </si>
@@ -983,7 +983,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B140"/>
+  <dimension ref="A1:B138"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -1972,15 +1972,15 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B124" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B125" t="s">
         <v>22</v>
@@ -1988,15 +1988,15 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="B126" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B127" t="s">
         <v>34</v>
@@ -2004,10 +2004,10 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="B128" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.35">
@@ -2015,7 +2015,7 @@
         <v>48</v>
       </c>
       <c r="B129" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.35">
@@ -2023,7 +2023,7 @@
         <v>48</v>
       </c>
       <c r="B130" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.35">
@@ -2031,7 +2031,7 @@
         <v>48</v>
       </c>
       <c r="B131" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.35">
@@ -2039,15 +2039,15 @@
         <v>48</v>
       </c>
       <c r="B132" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B133" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.35">
@@ -2055,7 +2055,7 @@
         <v>38</v>
       </c>
       <c r="B134" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.35">
@@ -2063,47 +2063,31 @@
         <v>38</v>
       </c>
       <c r="B135" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="B136" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
+        <v>20</v>
+      </c>
+      <c r="B137" t="s">
         <v>74</v>
-      </c>
-      <c r="B137" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
+        <v>77</v>
+      </c>
+      <c r="B138" t="s">
         <v>20</v>
-      </c>
-      <c r="B138" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A139" t="s">
-        <v>77</v>
-      </c>
-      <c r="B139" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A140" t="s">
-        <v>53</v>
-      </c>
-      <c r="B140" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -2113,7 +2097,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I277"/>
+  <dimension ref="A1:I275"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -5688,13 +5672,13 @@
         <v>11</v>
       </c>
       <c r="B124" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C124" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="D124">
-        <v>80.3</v>
+        <v>180.20050000000001</v>
       </c>
       <c r="E124">
         <v>500</v>
@@ -5717,13 +5701,13 @@
         <v>11</v>
       </c>
       <c r="B125" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C125" t="s">
         <v>22</v>
       </c>
       <c r="D125">
-        <v>180.20050000000001</v>
+        <v>421.21</v>
       </c>
       <c r="E125">
         <v>500</v>
@@ -5746,13 +5730,13 @@
         <v>11</v>
       </c>
       <c r="B126" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="C126" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D126">
-        <v>421.21</v>
+        <v>123.04150000000001</v>
       </c>
       <c r="E126">
         <v>500</v>
@@ -5775,13 +5759,13 @@
         <v>11</v>
       </c>
       <c r="B127" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C127" t="s">
         <v>34</v>
       </c>
       <c r="D127">
-        <v>123.04150000000001</v>
+        <v>161.62200000000001</v>
       </c>
       <c r="E127">
         <v>500</v>
@@ -5804,13 +5788,13 @@
         <v>11</v>
       </c>
       <c r="B128" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C128" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D128">
-        <v>161.62200000000001</v>
+        <v>455.15499999999997</v>
       </c>
       <c r="E128">
         <v>500</v>
@@ -5836,10 +5820,10 @@
         <v>48</v>
       </c>
       <c r="C129" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D129">
-        <v>455.15499999999997</v>
+        <v>351.714</v>
       </c>
       <c r="E129">
         <v>500</v>
@@ -5865,10 +5849,10 @@
         <v>48</v>
       </c>
       <c r="C130" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D130">
-        <v>351.714</v>
+        <v>167.75399999999999</v>
       </c>
       <c r="E130">
         <v>500</v>
@@ -5894,10 +5878,10 @@
         <v>48</v>
       </c>
       <c r="C131" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D131">
-        <v>167.75399999999999</v>
+        <v>207.5025</v>
       </c>
       <c r="E131">
         <v>500</v>
@@ -5923,10 +5907,10 @@
         <v>48</v>
       </c>
       <c r="C132" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D132">
-        <v>207.5025</v>
+        <v>513.19000000000005</v>
       </c>
       <c r="E132">
         <v>500</v>
@@ -5949,13 +5933,13 @@
         <v>11</v>
       </c>
       <c r="B133" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C133" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="D133">
-        <v>513.19000000000005</v>
+        <v>140.52500000000001</v>
       </c>
       <c r="E133">
         <v>500</v>
@@ -5981,10 +5965,10 @@
         <v>38</v>
       </c>
       <c r="C134" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="D134">
-        <v>140.52500000000001</v>
+        <v>82.927999999999997</v>
       </c>
       <c r="E134">
         <v>500</v>
@@ -6010,10 +5994,10 @@
         <v>38</v>
       </c>
       <c r="C135" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D135">
-        <v>82.927999999999997</v>
+        <v>67.451999999999998</v>
       </c>
       <c r="E135">
         <v>500</v>
@@ -6036,16 +6020,16 @@
         <v>11</v>
       </c>
       <c r="B136" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="C136" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D136">
-        <v>67.451999999999998</v>
+        <v>395</v>
       </c>
       <c r="E136">
-        <v>500</v>
+        <v>395</v>
       </c>
       <c r="F136">
         <v>1</v>
@@ -6065,10 +6049,10 @@
         <v>11</v>
       </c>
       <c r="B137" t="s">
+        <v>20</v>
+      </c>
+      <c r="C137" t="s">
         <v>74</v>
-      </c>
-      <c r="C137" t="s">
-        <v>22</v>
       </c>
       <c r="D137">
         <v>395</v>
@@ -6094,10 +6078,10 @@
         <v>11</v>
       </c>
       <c r="B138" t="s">
+        <v>77</v>
+      </c>
+      <c r="C138" t="s">
         <v>20</v>
-      </c>
-      <c r="C138" t="s">
-        <v>74</v>
       </c>
       <c r="D138">
         <v>395</v>
@@ -6120,19 +6104,19 @@
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B139" t="s">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="C139" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D139">
-        <v>395</v>
+        <v>500</v>
       </c>
       <c r="E139">
-        <v>395</v>
+        <v>500</v>
       </c>
       <c r="F139">
         <v>1</v>
@@ -6141,7 +6125,7 @@
         <v>10000000</v>
       </c>
       <c r="H139">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I139">
         <v>1</v>
@@ -6152,10 +6136,10 @@
         <v>12</v>
       </c>
       <c r="B140" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C140" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D140">
         <v>500</v>
@@ -6181,10 +6165,10 @@
         <v>12</v>
       </c>
       <c r="B141" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C141" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D141">
         <v>500</v>
@@ -6210,10 +6194,10 @@
         <v>12</v>
       </c>
       <c r="B142" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C142" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D142">
         <v>500</v>
@@ -6239,10 +6223,10 @@
         <v>12</v>
       </c>
       <c r="B143" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C143" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D143">
         <v>500</v>
@@ -6268,10 +6252,10 @@
         <v>12</v>
       </c>
       <c r="B144" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C144" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D144">
         <v>500</v>
@@ -6297,10 +6281,10 @@
         <v>12</v>
       </c>
       <c r="B145" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C145" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D145">
         <v>500</v>
@@ -6326,10 +6310,10 @@
         <v>12</v>
       </c>
       <c r="B146" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C146" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D146">
         <v>500</v>
@@ -6355,10 +6339,10 @@
         <v>12</v>
       </c>
       <c r="B147" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C147" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D147">
         <v>500</v>
@@ -6384,10 +6368,10 @@
         <v>12</v>
       </c>
       <c r="B148" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C148" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D148">
         <v>500</v>
@@ -6413,10 +6397,10 @@
         <v>12</v>
       </c>
       <c r="B149" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C149" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D149">
         <v>500</v>
@@ -6442,10 +6426,10 @@
         <v>12</v>
       </c>
       <c r="B150" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C150" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D150">
         <v>500</v>
@@ -6471,10 +6455,10 @@
         <v>12</v>
       </c>
       <c r="B151" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
       <c r="C151" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="D151">
         <v>500</v>
@@ -6500,10 +6484,10 @@
         <v>12</v>
       </c>
       <c r="B152" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="D152">
         <v>500</v>
@@ -6529,10 +6513,10 @@
         <v>12</v>
       </c>
       <c r="B153" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C153" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D153">
         <v>500</v>
@@ -6558,10 +6542,10 @@
         <v>12</v>
       </c>
       <c r="B154" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C154" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D154">
         <v>500</v>
@@ -6587,10 +6571,10 @@
         <v>12</v>
       </c>
       <c r="B155" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C155" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D155">
         <v>500</v>
@@ -6616,10 +6600,10 @@
         <v>12</v>
       </c>
       <c r="B156" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C156" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="D156">
         <v>500</v>
@@ -6645,10 +6629,10 @@
         <v>12</v>
       </c>
       <c r="B157" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C157" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D157">
         <v>500</v>
@@ -6674,10 +6658,10 @@
         <v>12</v>
       </c>
       <c r="B158" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C158" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="D158">
         <v>500</v>
@@ -6703,10 +6687,10 @@
         <v>12</v>
       </c>
       <c r="B159" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C159" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="D159">
         <v>500</v>
@@ -6732,10 +6716,10 @@
         <v>12</v>
       </c>
       <c r="B160" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C160" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D160">
         <v>500</v>
@@ -6761,10 +6745,10 @@
         <v>12</v>
       </c>
       <c r="B161" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C161" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D161">
         <v>500</v>
@@ -6790,10 +6774,10 @@
         <v>12</v>
       </c>
       <c r="B162" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C162" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="D162">
         <v>500</v>
@@ -6819,10 +6803,10 @@
         <v>12</v>
       </c>
       <c r="B163" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C163" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="D163">
         <v>500</v>
@@ -6848,10 +6832,10 @@
         <v>12</v>
       </c>
       <c r="B164" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="C164" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="D164">
         <v>500</v>
@@ -6880,7 +6864,7 @@
         <v>38</v>
       </c>
       <c r="C165" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="D165">
         <v>500</v>
@@ -6906,10 +6890,10 @@
         <v>12</v>
       </c>
       <c r="B166" t="s">
+        <v>16</v>
+      </c>
+      <c r="C166" t="s">
         <v>38</v>
-      </c>
-      <c r="C166" t="s">
-        <v>59</v>
       </c>
       <c r="D166">
         <v>500</v>
@@ -6938,7 +6922,7 @@
         <v>16</v>
       </c>
       <c r="C167" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="D167">
         <v>500</v>
@@ -6967,7 +6951,7 @@
         <v>16</v>
       </c>
       <c r="C168" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D168">
         <v>500</v>
@@ -6996,7 +6980,7 @@
         <v>16</v>
       </c>
       <c r="C169" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="D169">
         <v>500</v>
@@ -7022,10 +7006,10 @@
         <v>12</v>
       </c>
       <c r="B170" t="s">
+        <v>28</v>
+      </c>
+      <c r="C170" t="s">
         <v>16</v>
-      </c>
-      <c r="C170" t="s">
-        <v>18</v>
       </c>
       <c r="D170">
         <v>500</v>
@@ -7054,7 +7038,7 @@
         <v>28</v>
       </c>
       <c r="C171" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D171">
         <v>500</v>
@@ -7080,10 +7064,10 @@
         <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="C172" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D172">
         <v>500</v>
@@ -7112,7 +7096,7 @@
         <v>42</v>
       </c>
       <c r="C173" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D173">
         <v>500</v>
@@ -7141,7 +7125,7 @@
         <v>42</v>
       </c>
       <c r="C174" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="D174">
         <v>500</v>
@@ -7170,7 +7154,7 @@
         <v>42</v>
       </c>
       <c r="C175" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D175">
         <v>500</v>
@@ -7199,7 +7183,7 @@
         <v>42</v>
       </c>
       <c r="C176" t="s">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="D176">
         <v>500</v>
@@ -7228,7 +7212,7 @@
         <v>42</v>
       </c>
       <c r="C177" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D177">
         <v>500</v>
@@ -7257,7 +7241,7 @@
         <v>42</v>
       </c>
       <c r="C178" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D178">
         <v>500</v>
@@ -7286,7 +7270,7 @@
         <v>42</v>
       </c>
       <c r="C179" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="D179">
         <v>500</v>
@@ -7315,7 +7299,7 @@
         <v>42</v>
       </c>
       <c r="C180" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D180">
         <v>500</v>
@@ -7341,10 +7325,10 @@
         <v>12</v>
       </c>
       <c r="B181" t="s">
+        <v>60</v>
+      </c>
+      <c r="C181" t="s">
         <v>42</v>
-      </c>
-      <c r="C181" t="s">
-        <v>63</v>
       </c>
       <c r="D181">
         <v>500</v>
@@ -7373,7 +7357,7 @@
         <v>60</v>
       </c>
       <c r="C182" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D182">
         <v>500</v>
@@ -7402,7 +7386,7 @@
         <v>60</v>
       </c>
       <c r="C183" t="s">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="D183">
         <v>500</v>
@@ -7431,7 +7415,7 @@
         <v>60</v>
       </c>
       <c r="C184" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D184">
         <v>500</v>
@@ -7460,7 +7444,7 @@
         <v>60</v>
       </c>
       <c r="C185" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D185">
         <v>500</v>
@@ -7486,10 +7470,10 @@
         <v>12</v>
       </c>
       <c r="B186" t="s">
+        <v>22</v>
+      </c>
+      <c r="C186" t="s">
         <v>60</v>
-      </c>
-      <c r="C186" t="s">
-        <v>66</v>
       </c>
       <c r="D186">
         <v>500</v>
@@ -7518,7 +7502,7 @@
         <v>22</v>
       </c>
       <c r="C187" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D187">
         <v>500</v>
@@ -7547,7 +7531,7 @@
         <v>22</v>
       </c>
       <c r="C188" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D188">
         <v>500</v>
@@ -7573,10 +7557,10 @@
         <v>12</v>
       </c>
       <c r="B189" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="C189" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D189">
         <v>500</v>
@@ -7605,7 +7589,7 @@
         <v>61</v>
       </c>
       <c r="C190" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D190">
         <v>500</v>
@@ -7634,7 +7618,7 @@
         <v>61</v>
       </c>
       <c r="C191" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D191">
         <v>500</v>
@@ -7660,10 +7644,10 @@
         <v>12</v>
       </c>
       <c r="B192" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C192" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D192">
         <v>500</v>
@@ -7692,7 +7676,7 @@
         <v>64</v>
       </c>
       <c r="C193" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D193">
         <v>500</v>
@@ -7718,10 +7702,10 @@
         <v>12</v>
       </c>
       <c r="B194" t="s">
+        <v>24</v>
+      </c>
+      <c r="C194" t="s">
         <v>64</v>
-      </c>
-      <c r="C194" t="s">
-        <v>24</v>
       </c>
       <c r="D194">
         <v>500</v>
@@ -7750,7 +7734,7 @@
         <v>24</v>
       </c>
       <c r="C195" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D195">
         <v>500</v>
@@ -7776,10 +7760,10 @@
         <v>12</v>
       </c>
       <c r="B196" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C196" t="s">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="D196">
         <v>500</v>
@@ -7808,7 +7792,7 @@
         <v>18</v>
       </c>
       <c r="C197" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
       <c r="D197">
         <v>500</v>
@@ -7837,7 +7821,7 @@
         <v>18</v>
       </c>
       <c r="C198" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D198">
         <v>500</v>
@@ -7863,10 +7847,10 @@
         <v>12</v>
       </c>
       <c r="B199" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D199">
         <v>500</v>
@@ -7892,7 +7876,7 @@
         <v>12</v>
       </c>
       <c r="B200" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C200" t="s">
         <v>42</v>
@@ -7921,7 +7905,7 @@
         <v>12</v>
       </c>
       <c r="B201" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="C201" t="s">
         <v>42</v>
@@ -7953,7 +7937,7 @@
         <v>62</v>
       </c>
       <c r="C202" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D202">
         <v>500</v>
@@ -7982,7 +7966,7 @@
         <v>62</v>
       </c>
       <c r="C203" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="D203">
         <v>500</v>
@@ -8008,10 +7992,10 @@
         <v>12</v>
       </c>
       <c r="B204" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C204" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D204">
         <v>500</v>
@@ -8040,7 +8024,7 @@
         <v>65</v>
       </c>
       <c r="C205" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D205">
         <v>500</v>
@@ -8069,7 +8053,7 @@
         <v>65</v>
       </c>
       <c r="C206" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D206">
         <v>500</v>
@@ -8098,7 +8082,7 @@
         <v>65</v>
       </c>
       <c r="C207" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D207">
         <v>500</v>
@@ -8124,10 +8108,10 @@
         <v>12</v>
       </c>
       <c r="B208" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C208" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="D208">
         <v>500</v>
@@ -8156,7 +8140,7 @@
         <v>66</v>
       </c>
       <c r="C209" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D209">
         <v>500</v>
@@ -8185,7 +8169,7 @@
         <v>66</v>
       </c>
       <c r="C210" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D210">
         <v>500</v>
@@ -8214,7 +8198,7 @@
         <v>66</v>
       </c>
       <c r="C211" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="D211">
         <v>500</v>
@@ -8240,10 +8224,10 @@
         <v>12</v>
       </c>
       <c r="B212" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C212" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="D212">
         <v>500</v>
@@ -8272,7 +8256,7 @@
         <v>67</v>
       </c>
       <c r="C213" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D213">
         <v>500</v>
@@ -8298,10 +8282,10 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
+        <v>68</v>
+      </c>
+      <c r="C214" t="s">
         <v>67</v>
-      </c>
-      <c r="C214" t="s">
-        <v>69</v>
       </c>
       <c r="D214">
         <v>500</v>
@@ -8330,7 +8314,7 @@
         <v>68</v>
       </c>
       <c r="C215" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="D215">
         <v>500</v>
@@ -8359,7 +8343,7 @@
         <v>68</v>
       </c>
       <c r="C216" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="D216">
         <v>500</v>
@@ -8388,7 +8372,7 @@
         <v>68</v>
       </c>
       <c r="C217" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="D217">
         <v>500</v>
@@ -8417,7 +8401,7 @@
         <v>68</v>
       </c>
       <c r="C218" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="D218">
         <v>500</v>
@@ -8443,10 +8427,10 @@
         <v>12</v>
       </c>
       <c r="B219" t="s">
+        <v>20</v>
+      </c>
+      <c r="C219" t="s">
         <v>68</v>
-      </c>
-      <c r="C219" t="s">
-        <v>36</v>
       </c>
       <c r="D219">
         <v>500</v>
@@ -8472,10 +8456,10 @@
         <v>12</v>
       </c>
       <c r="B220" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C220" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D220">
         <v>500</v>
@@ -8504,7 +8488,7 @@
         <v>51</v>
       </c>
       <c r="C221" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D221">
         <v>500</v>
@@ -8533,7 +8517,7 @@
         <v>51</v>
       </c>
       <c r="C222" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D222">
         <v>500</v>
@@ -8562,7 +8546,7 @@
         <v>51</v>
       </c>
       <c r="C223" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="D223">
         <v>500</v>
@@ -8588,10 +8572,10 @@
         <v>12</v>
       </c>
       <c r="B224" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="C224" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D224">
         <v>500</v>
@@ -8620,7 +8604,7 @@
         <v>26</v>
       </c>
       <c r="C225" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="D225">
         <v>500</v>
@@ -8646,10 +8630,10 @@
         <v>12</v>
       </c>
       <c r="B226" t="s">
+        <v>72</v>
+      </c>
+      <c r="C226" t="s">
         <v>26</v>
-      </c>
-      <c r="C226" t="s">
-        <v>53</v>
       </c>
       <c r="D226">
         <v>500</v>
@@ -8678,7 +8662,7 @@
         <v>72</v>
       </c>
       <c r="C227" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="D227">
         <v>500</v>
@@ -8704,10 +8688,10 @@
         <v>12</v>
       </c>
       <c r="B228" t="s">
-        <v>72</v>
+        <v>34</v>
       </c>
       <c r="C228" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="D228">
         <v>500</v>
@@ -8736,7 +8720,7 @@
         <v>34</v>
       </c>
       <c r="C229" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D229">
         <v>500</v>
@@ -8762,10 +8746,10 @@
         <v>12</v>
       </c>
       <c r="B230" t="s">
+        <v>32</v>
+      </c>
+      <c r="C230" t="s">
         <v>34</v>
-      </c>
-      <c r="C230" t="s">
-        <v>32</v>
       </c>
       <c r="D230">
         <v>500</v>
@@ -8791,10 +8775,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C231" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D231">
         <v>500</v>
@@ -8823,7 +8807,7 @@
         <v>58</v>
       </c>
       <c r="C232" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="D232">
         <v>500</v>
@@ -8852,7 +8836,7 @@
         <v>58</v>
       </c>
       <c r="C233" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D233">
         <v>500</v>
@@ -8881,7 +8865,7 @@
         <v>58</v>
       </c>
       <c r="C234" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="D234">
         <v>500</v>
@@ -8907,7 +8891,7 @@
         <v>12</v>
       </c>
       <c r="B235" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="C235" t="s">
         <v>51</v>
@@ -8936,10 +8920,10 @@
         <v>12</v>
       </c>
       <c r="B236" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="C236" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D236">
         <v>500</v>
@@ -8968,7 +8952,7 @@
         <v>53</v>
       </c>
       <c r="C237" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="D237">
         <v>500</v>
@@ -8997,7 +8981,7 @@
         <v>53</v>
       </c>
       <c r="C238" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D238">
         <v>500</v>
@@ -9023,10 +9007,10 @@
         <v>12</v>
       </c>
       <c r="B239" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="C239" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="D239">
         <v>500</v>
@@ -9052,10 +9036,10 @@
         <v>12</v>
       </c>
       <c r="B240" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="C240" t="s">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="D240">
         <v>500</v>
@@ -9084,7 +9068,7 @@
         <v>36</v>
       </c>
       <c r="C241" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="D241">
         <v>500</v>
@@ -9110,10 +9094,10 @@
         <v>12</v>
       </c>
       <c r="B242" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C242" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="D242">
         <v>500</v>
@@ -9142,7 +9126,7 @@
         <v>48</v>
       </c>
       <c r="C243" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="D243">
         <v>500</v>
@@ -9171,7 +9155,7 @@
         <v>48</v>
       </c>
       <c r="C244" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D244">
         <v>500</v>
@@ -9200,7 +9184,7 @@
         <v>48</v>
       </c>
       <c r="C245" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="D245">
         <v>500</v>
@@ -9226,10 +9210,10 @@
         <v>12</v>
       </c>
       <c r="B246" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="C246" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="D246">
         <v>500</v>
@@ -9255,10 +9239,10 @@
         <v>12</v>
       </c>
       <c r="B247" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="C247" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="D247">
         <v>500</v>
@@ -9284,7 +9268,7 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C248" t="s">
         <v>22</v>
@@ -9313,10 +9297,10 @@
         <v>12</v>
       </c>
       <c r="B249" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="C249" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D249">
         <v>500</v>
@@ -9345,7 +9329,7 @@
         <v>75</v>
       </c>
       <c r="C250" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D250">
         <v>500</v>
@@ -9371,10 +9355,10 @@
         <v>12</v>
       </c>
       <c r="B251" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C251" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="D251">
         <v>500</v>
@@ -9400,10 +9384,10 @@
         <v>12</v>
       </c>
       <c r="B252" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C252" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="D252">
         <v>500</v>
@@ -9429,10 +9413,10 @@
         <v>12</v>
       </c>
       <c r="B253" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="C253" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="D253">
         <v>500</v>
@@ -9461,7 +9445,7 @@
         <v>58</v>
       </c>
       <c r="C254" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="D254">
         <v>500</v>
@@ -9490,7 +9474,7 @@
         <v>58</v>
       </c>
       <c r="C255" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D255">
         <v>500</v>
@@ -9516,7 +9500,7 @@
         <v>12</v>
       </c>
       <c r="B256" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="C256" t="s">
         <v>66</v>
@@ -9545,10 +9529,10 @@
         <v>12</v>
       </c>
       <c r="B257" t="s">
+        <v>68</v>
+      </c>
+      <c r="C257" t="s">
         <v>67</v>
-      </c>
-      <c r="C257" t="s">
-        <v>66</v>
       </c>
       <c r="D257">
         <v>500</v>
@@ -9577,7 +9561,7 @@
         <v>68</v>
       </c>
       <c r="C258" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D258">
         <v>500</v>
@@ -9603,10 +9587,10 @@
         <v>12</v>
       </c>
       <c r="B259" t="s">
+        <v>36</v>
+      </c>
+      <c r="C259" t="s">
         <v>68</v>
-      </c>
-      <c r="C259" t="s">
-        <v>70</v>
       </c>
       <c r="D259">
         <v>500</v>
@@ -9632,10 +9616,10 @@
         <v>12</v>
       </c>
       <c r="B260" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="C260" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D260">
         <v>500</v>
@@ -9661,10 +9645,10 @@
         <v>12</v>
       </c>
       <c r="B261" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C261" t="s">
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="D261">
         <v>500</v>
@@ -9690,10 +9674,10 @@
         <v>12</v>
       </c>
       <c r="B262" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C262" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="D262">
         <v>500</v>
@@ -9719,10 +9703,10 @@
         <v>12</v>
       </c>
       <c r="B263" t="s">
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="C263" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D263">
         <v>500</v>
@@ -9748,10 +9732,10 @@
         <v>12</v>
       </c>
       <c r="B264" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C264" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D264">
         <v>500</v>
@@ -9777,10 +9761,10 @@
         <v>12</v>
       </c>
       <c r="B265" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="C265" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D265">
         <v>500</v>
@@ -9806,10 +9790,10 @@
         <v>12</v>
       </c>
       <c r="B266" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C266" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D266">
         <v>500</v>
@@ -9838,7 +9822,7 @@
         <v>48</v>
       </c>
       <c r="C267" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D267">
         <v>500</v>
@@ -9867,7 +9851,7 @@
         <v>48</v>
       </c>
       <c r="C268" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D268">
         <v>500</v>
@@ -9896,7 +9880,7 @@
         <v>48</v>
       </c>
       <c r="C269" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D269">
         <v>500</v>
@@ -9922,10 +9906,10 @@
         <v>12</v>
       </c>
       <c r="B270" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C270" t="s">
-        <v>18</v>
+        <v>79</v>
       </c>
       <c r="D270">
         <v>500</v>
@@ -9951,10 +9935,10 @@
         <v>12</v>
       </c>
       <c r="B271" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C271" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="D271">
         <v>500</v>
@@ -9983,7 +9967,7 @@
         <v>38</v>
       </c>
       <c r="C272" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="D272">
         <v>500</v>
@@ -10009,10 +9993,10 @@
         <v>12</v>
       </c>
       <c r="B273" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="C273" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D273">
         <v>500</v>
@@ -10038,10 +10022,10 @@
         <v>12</v>
       </c>
       <c r="B274" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="C274" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="D274">
         <v>500</v>
@@ -10067,10 +10051,10 @@
         <v>12</v>
       </c>
       <c r="B275" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C275" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D275">
         <v>500</v>
@@ -10088,64 +10072,6 @@
         <v>1000</v>
       </c>
       <c r="I275">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A276" t="s">
-        <v>12</v>
-      </c>
-      <c r="B276" t="s">
-        <v>20</v>
-      </c>
-      <c r="C276" t="s">
-        <v>74</v>
-      </c>
-      <c r="D276">
-        <v>500</v>
-      </c>
-      <c r="E276">
-        <v>500</v>
-      </c>
-      <c r="F276">
-        <v>1</v>
-      </c>
-      <c r="G276">
-        <v>10000000</v>
-      </c>
-      <c r="H276">
-        <v>1000</v>
-      </c>
-      <c r="I276">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A277" t="s">
-        <v>12</v>
-      </c>
-      <c r="B277" t="s">
-        <v>77</v>
-      </c>
-      <c r="C277" t="s">
-        <v>20</v>
-      </c>
-      <c r="D277">
-        <v>500</v>
-      </c>
-      <c r="E277">
-        <v>500</v>
-      </c>
-      <c r="F277">
-        <v>1</v>
-      </c>
-      <c r="G277">
-        <v>10000000</v>
-      </c>
-      <c r="H277">
-        <v>1000</v>
-      </c>
-      <c r="I277">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update gas production in Europe for Russian case
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F33ECF1-A089-4749-A056-AEFBEFD9B9AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0496360A-C275-4DAC-8138-12AE6D08D54C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1424" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1537" uniqueCount="99">
   <si>
     <t>Commodities</t>
   </si>
@@ -286,6 +286,57 @@
   </si>
   <si>
     <t>SE</t>
+  </si>
+  <si>
+    <t>AL_Prod</t>
+  </si>
+  <si>
+    <t>DZ_Prod</t>
+  </si>
+  <si>
+    <t>DZ</t>
+  </si>
+  <si>
+    <t>AT_Prod</t>
+  </si>
+  <si>
+    <t>BE_Prod</t>
+  </si>
+  <si>
+    <t>BG_Prod</t>
+  </si>
+  <si>
+    <t>HR_Prod</t>
+  </si>
+  <si>
+    <t>CZ_Prod</t>
+  </si>
+  <si>
+    <t>FR_Prod</t>
+  </si>
+  <si>
+    <t>GR_Prod</t>
+  </si>
+  <si>
+    <t>HU_Prod</t>
+  </si>
+  <si>
+    <t>IE_Prod</t>
+  </si>
+  <si>
+    <t>RS_Prod</t>
+  </si>
+  <si>
+    <t>SK_Prod</t>
+  </si>
+  <si>
+    <t>SI_Prod</t>
+  </si>
+  <si>
+    <t>TR_Prod</t>
+  </si>
+  <si>
+    <t>ES_Prod</t>
   </si>
 </sst>
 </file>
@@ -643,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B0CB446-BDDD-415D-AF22-2CEB1FE45CA5}">
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A78"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -949,6 +1000,91 @@
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -983,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B138"/>
+  <dimension ref="A1:B154"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -1988,7 +2124,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B126" t="s">
         <v>34</v>
@@ -2088,6 +2224,134 @@
       </c>
       <c r="B138" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>82</v>
+      </c>
+      <c r="B139" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>83</v>
+      </c>
+      <c r="B140" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>85</v>
+      </c>
+      <c r="B141" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>86</v>
+      </c>
+      <c r="B142" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>87</v>
+      </c>
+      <c r="B143" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>88</v>
+      </c>
+      <c r="B144" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>89</v>
+      </c>
+      <c r="B145" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>90</v>
+      </c>
+      <c r="B146" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>91</v>
+      </c>
+      <c r="B147" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>92</v>
+      </c>
+      <c r="B148" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>93</v>
+      </c>
+      <c r="B149" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>94</v>
+      </c>
+      <c r="B150" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>95</v>
+      </c>
+      <c r="B151" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>96</v>
+      </c>
+      <c r="B152" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>97</v>
+      </c>
+      <c r="B153" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>98</v>
+      </c>
+      <c r="B154" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -10083,7 +10347,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68B577B-1347-43AB-A697-F4519763B965}">
-  <dimension ref="A1:G125"/>
+  <dimension ref="A1:G157"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -10245,10 +10509,10 @@
         <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="C15">
-        <v>13.677999999999999</v>
+        <v>0.55586415</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -10256,10 +10520,10 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="C16">
-        <v>43.964999999999996</v>
+        <v>796.255</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -10267,10 +10531,10 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="C17">
-        <v>38.102999999999994</v>
+        <v>7.5617455199999997</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -10278,10 +10542,10 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="C18">
-        <v>129.941</v>
+        <v>5.7643000000000007E-2</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -10289,10 +10553,10 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="C19">
-        <v>195.39999999999998</v>
+        <v>0.53100926999999998</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -10300,10 +10564,10 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>88</v>
       </c>
       <c r="C20">
-        <v>1089.355</v>
+        <v>8.6795214499999993</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -10311,10 +10575,10 @@
         <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>89</v>
       </c>
       <c r="C21">
-        <v>38.102999999999994</v>
+        <v>1.9156527500000002</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -10322,10 +10586,10 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C22">
-        <v>84.998999999999995</v>
+        <v>0.16949973000000002</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -10333,10 +10597,10 @@
         <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="C23">
-        <v>6238.1449999999995</v>
+        <v>6.3309600000000021E-2</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -10344,10 +10608,10 @@
         <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="C24">
-        <v>18.562999999999999</v>
+        <v>16.46245</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -10355,10 +10619,10 @@
         <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="C25">
-        <v>385.91499999999996</v>
+        <v>19.829690269999997</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -10366,10 +10630,10 @@
         <v>11</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="C26">
-        <v>185.63</v>
+        <v>3.9959299999999995</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -10377,10 +10641,10 @@
         <v>11</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>95</v>
       </c>
       <c r="C27">
-        <v>-708.32499999999993</v>
+        <v>0.6516687699999999</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -10388,10 +10652,10 @@
         <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>16</v>
+        <v>96</v>
       </c>
       <c r="C28">
-        <v>-166.09</v>
+        <v>5.2113180000000002E-2</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -10399,10 +10663,10 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="C29">
-        <v>-357.58199999999999</v>
+        <v>4.2744726999999996</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -10410,10 +10674,10 @@
         <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="C30">
-        <v>-845.10500000000002</v>
+        <v>0.44941999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
@@ -10421,10 +10685,10 @@
         <v>11</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="C31">
-        <v>-83.045000000000002</v>
+        <v>13.947075569999997</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -10432,426 +10696,426 @@
         <v>11</v>
       </c>
       <c r="B32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32">
+        <v>47.618979999999993</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33">
+        <v>38.415639999999996</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34">
+        <v>129.941</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35">
+        <v>234.14902171</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36">
+        <v>1135.3337630899998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37">
+        <v>54.642437600000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38">
+        <v>88.09608999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39">
+        <v>6238.1449999999995</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" t="s">
+        <v>54</v>
+      </c>
+      <c r="C40">
+        <v>18.562999999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41">
+        <v>320.81311303999996</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42">
+        <v>190.67131999999998</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" t="s">
+        <v>38</v>
+      </c>
+      <c r="C43">
+        <v>-708.32499999999993</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>11</v>
+      </c>
+      <c r="B44" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44">
+        <v>-166.09</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>11</v>
+      </c>
+      <c r="B45" t="s">
+        <v>28</v>
+      </c>
+      <c r="C45">
+        <v>-357.58199999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" t="s">
+        <v>42</v>
+      </c>
+      <c r="C46">
+        <v>-845.10500000000002</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" t="s">
+        <v>60</v>
+      </c>
+      <c r="C47">
+        <v>-83.045000000000002</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>11</v>
+      </c>
+      <c r="B48" t="s">
         <v>22</v>
       </c>
-      <c r="C32">
+      <c r="C48">
         <v>-661.42899999999997</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>11</v>
-      </c>
-      <c r="B33" t="s">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>11</v>
+      </c>
+      <c r="B49" t="s">
         <v>61</v>
       </c>
-      <c r="C33">
+      <c r="C49">
         <v>-31.263999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34" t="s">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>11</v>
+      </c>
+      <c r="B50" t="s">
         <v>64</v>
       </c>
-      <c r="C34">
+      <c r="C50">
         <v>-30</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" t="s">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>11</v>
+      </c>
+      <c r="B51" t="s">
         <v>24</v>
       </c>
-      <c r="C35">
+      <c r="C51">
         <v>-50</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" t="s">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>11</v>
+      </c>
+      <c r="B52" t="s">
         <v>18</v>
       </c>
-      <c r="C36">
+      <c r="C52">
         <v>-397.63900000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>11</v>
-      </c>
-      <c r="B37" t="s">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>11</v>
+      </c>
+      <c r="B53" t="s">
         <v>40</v>
       </c>
-      <c r="C37">
+      <c r="C53">
         <v>-100</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>11</v>
-      </c>
-      <c r="B38" t="s">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>11</v>
+      </c>
+      <c r="B54" t="s">
         <v>30</v>
       </c>
-      <c r="C38">
+      <c r="C54">
         <v>-211.03200000000001</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F54" t="s">
         <v>81</v>
       </c>
-      <c r="G38">
+      <c r="G54">
         <v>-10.747</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>11</v>
-      </c>
-      <c r="B39" t="s">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>11</v>
+      </c>
+      <c r="B55" t="s">
         <v>62</v>
       </c>
-      <c r="C39">
+      <c r="C55">
         <v>-83.045000000000002</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F55" t="s">
         <v>77</v>
       </c>
-      <c r="G39">
+      <c r="G55">
         <v>-453.32799999999997</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>11</v>
-      </c>
-      <c r="B40" t="s">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>11</v>
+      </c>
+      <c r="B56" t="s">
         <v>65</v>
       </c>
-      <c r="C40">
+      <c r="C56">
         <v>-30</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>11</v>
-      </c>
-      <c r="B41" t="s">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>11</v>
+      </c>
+      <c r="B57" t="s">
         <v>66</v>
       </c>
-      <c r="C41">
+      <c r="C57">
         <v>-99.653999999999982</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>11</v>
-      </c>
-      <c r="B42" t="s">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>11</v>
+      </c>
+      <c r="B58" t="s">
         <v>67</v>
       </c>
-      <c r="C42">
+      <c r="C58">
         <v>-30</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" t="s">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>11</v>
+      </c>
+      <c r="B59" t="s">
         <v>73</v>
       </c>
-      <c r="C43">
+      <c r="C59">
         <v>-19.54</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>11</v>
-      </c>
-      <c r="B44" t="s">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>11</v>
+      </c>
+      <c r="B60" t="s">
         <v>68</v>
       </c>
-      <c r="C44">
+      <c r="C60">
         <v>-50</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>11</v>
-      </c>
-      <c r="B45" t="s">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>11</v>
+      </c>
+      <c r="B61" t="s">
         <v>20</v>
       </c>
-      <c r="C45">
+      <c r="C61">
         <v>-55.689</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>11</v>
-      </c>
-      <c r="B46" t="s">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>11</v>
+      </c>
+      <c r="B62" t="s">
         <v>51</v>
       </c>
-      <c r="C46">
+      <c r="C62">
         <v>-110.401</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>11</v>
-      </c>
-      <c r="B47" t="s">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>11</v>
+      </c>
+      <c r="B63" t="s">
         <v>26</v>
       </c>
-      <c r="C47">
+      <c r="C63">
         <v>-20</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>11</v>
-      </c>
-      <c r="B48" t="s">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>11</v>
+      </c>
+      <c r="B64" t="s">
         <v>72</v>
       </c>
-      <c r="C48">
+      <c r="C64">
         <v>-20</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>11</v>
-      </c>
-      <c r="B49" t="s">
-        <v>34</v>
-      </c>
-      <c r="C49">
-        <v>-316.54799999999994</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>11</v>
-      </c>
-      <c r="B50" t="s">
-        <v>32</v>
-      </c>
-      <c r="C50">
-        <v>-58.62</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>11</v>
-      </c>
-      <c r="B51" t="s">
-        <v>58</v>
-      </c>
-      <c r="C51">
-        <v>-286.26099999999997</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>11</v>
-      </c>
-      <c r="B52" t="s">
-        <v>71</v>
-      </c>
-      <c r="C52">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>11</v>
-      </c>
-      <c r="B53" t="s">
-        <v>53</v>
-      </c>
-      <c r="C53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>11</v>
-      </c>
-      <c r="B54" t="s">
-        <v>74</v>
-      </c>
-      <c r="C54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>11</v>
-      </c>
-      <c r="B55" t="s">
-        <v>36</v>
-      </c>
-      <c r="C55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>11</v>
-      </c>
-      <c r="B56" t="s">
-        <v>48</v>
-      </c>
-      <c r="C56">
-        <v>-42.988</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>11</v>
-      </c>
-      <c r="B57" t="s">
-        <v>78</v>
-      </c>
-      <c r="C57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>11</v>
-      </c>
-      <c r="B58" t="s">
-        <v>55</v>
-      </c>
-      <c r="C58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>11</v>
-      </c>
-      <c r="B59" t="s">
-        <v>45</v>
-      </c>
-      <c r="C59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>11</v>
-      </c>
-      <c r="B60" t="s">
-        <v>75</v>
-      </c>
-      <c r="C60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>11</v>
-      </c>
-      <c r="B61" t="s">
-        <v>76</v>
-      </c>
-      <c r="C61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>11</v>
-      </c>
-      <c r="B62" t="s">
-        <v>78</v>
-      </c>
-      <c r="C62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>12</v>
-      </c>
-      <c r="B63" t="s">
-        <v>15</v>
-      </c>
-      <c r="C63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>12</v>
-      </c>
-      <c r="B64" t="s">
-        <v>17</v>
-      </c>
-      <c r="C64">
-        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B65" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="C65">
-        <v>0</v>
+        <v>-316.54799999999994</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C66">
-        <v>0</v>
+        <v>-58.62</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B67" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="C67">
-        <v>0</v>
+        <v>-286.26099999999997</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="C68">
-        <v>0</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -10859,10 +11123,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B70" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -10870,10 +11134,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B71" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -10881,21 +11145,21 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B72" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="C72">
-        <v>0</v>
+        <v>-42.988</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B73" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="C73">
         <v>0</v>
@@ -10903,10 +11167,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="C74">
         <v>0</v>
@@ -10914,10 +11178,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="C75">
         <v>0</v>
@@ -10925,10 +11189,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B76" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="C76">
         <v>0</v>
@@ -10936,10 +11200,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B77" t="s">
-        <v>41</v>
+        <v>76</v>
       </c>
       <c r="C77">
         <v>0</v>
@@ -10947,10 +11211,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B78" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -10961,7 +11225,7 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -10972,7 +11236,7 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="C80">
         <v>0</v>
@@ -10983,7 +11247,7 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="C81">
         <v>0</v>
@@ -10994,7 +11258,7 @@
         <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="C82">
         <v>0</v>
@@ -11005,7 +11269,7 @@
         <v>12</v>
       </c>
       <c r="B83" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="C83">
         <v>0</v>
@@ -11016,7 +11280,7 @@
         <v>12</v>
       </c>
       <c r="B84" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -11027,7 +11291,7 @@
         <v>12</v>
       </c>
       <c r="B85" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -11038,7 +11302,7 @@
         <v>12</v>
       </c>
       <c r="B86" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -11049,7 +11313,7 @@
         <v>12</v>
       </c>
       <c r="B87" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -11060,7 +11324,7 @@
         <v>12</v>
       </c>
       <c r="B88" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -11071,7 +11335,7 @@
         <v>12</v>
       </c>
       <c r="B89" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -11082,7 +11346,7 @@
         <v>12</v>
       </c>
       <c r="B90" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -11093,7 +11357,7 @@
         <v>12</v>
       </c>
       <c r="B91" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -11104,7 +11368,7 @@
         <v>12</v>
       </c>
       <c r="B92" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -11115,7 +11379,7 @@
         <v>12</v>
       </c>
       <c r="B93" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -11126,7 +11390,7 @@
         <v>12</v>
       </c>
       <c r="B94" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="C94">
         <v>0</v>
@@ -11137,7 +11401,7 @@
         <v>12</v>
       </c>
       <c r="B95" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="C95">
         <v>0</v>
@@ -11148,7 +11412,7 @@
         <v>12</v>
       </c>
       <c r="B96" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="C96">
         <v>0</v>
@@ -11159,7 +11423,7 @@
         <v>12</v>
       </c>
       <c r="B97" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C97">
         <v>0</v>
@@ -11170,7 +11434,7 @@
         <v>12</v>
       </c>
       <c r="B98" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C98">
         <v>0</v>
@@ -11181,7 +11445,7 @@
         <v>12</v>
       </c>
       <c r="B99" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C99">
         <v>0</v>
@@ -11192,7 +11456,7 @@
         <v>12</v>
       </c>
       <c r="B100" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C100">
         <v>0</v>
@@ -11203,7 +11467,7 @@
         <v>12</v>
       </c>
       <c r="B101" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="C101">
         <v>0</v>
@@ -11214,7 +11478,7 @@
         <v>12</v>
       </c>
       <c r="B102" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C102">
         <v>0</v>
@@ -11225,7 +11489,7 @@
         <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C103">
         <v>0</v>
@@ -11236,7 +11500,7 @@
         <v>12</v>
       </c>
       <c r="B104" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="C104">
         <v>0</v>
@@ -11247,7 +11511,7 @@
         <v>12</v>
       </c>
       <c r="B105" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C105">
         <v>0</v>
@@ -11258,7 +11522,7 @@
         <v>12</v>
       </c>
       <c r="B106" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C106">
         <v>0</v>
@@ -11269,7 +11533,7 @@
         <v>12</v>
       </c>
       <c r="B107" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="C107">
         <v>0</v>
@@ -11280,7 +11544,7 @@
         <v>12</v>
       </c>
       <c r="B108" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -11291,7 +11555,7 @@
         <v>12</v>
       </c>
       <c r="B109" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -11302,7 +11566,7 @@
         <v>12</v>
       </c>
       <c r="B110" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -11313,7 +11577,7 @@
         <v>12</v>
       </c>
       <c r="B111" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -11324,7 +11588,7 @@
         <v>12</v>
       </c>
       <c r="B112" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -11335,7 +11599,7 @@
         <v>12</v>
       </c>
       <c r="B113" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -11346,7 +11610,7 @@
         <v>12</v>
       </c>
       <c r="B114" t="s">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -11357,7 +11621,7 @@
         <v>12</v>
       </c>
       <c r="B115" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -11368,7 +11632,7 @@
         <v>12</v>
       </c>
       <c r="B116" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C116">
         <v>0</v>
@@ -11379,7 +11643,7 @@
         <v>12</v>
       </c>
       <c r="B117" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="C117">
         <v>0</v>
@@ -11390,7 +11654,7 @@
         <v>12</v>
       </c>
       <c r="B118" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="C118">
         <v>0</v>
@@ -11401,7 +11665,7 @@
         <v>12</v>
       </c>
       <c r="B119" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C119">
         <v>0</v>
@@ -11412,7 +11676,7 @@
         <v>12</v>
       </c>
       <c r="B120" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C120">
         <v>0</v>
@@ -11423,7 +11687,7 @@
         <v>12</v>
       </c>
       <c r="B121" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="C121">
         <v>0</v>
@@ -11434,7 +11698,7 @@
         <v>12</v>
       </c>
       <c r="B122" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="C122">
         <v>0</v>
@@ -11442,10 +11706,10 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B123" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="C123">
         <v>0</v>
@@ -11456,7 +11720,7 @@
         <v>12</v>
       </c>
       <c r="B124" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C124">
         <v>0</v>
@@ -11467,9 +11731,361 @@
         <v>12</v>
       </c>
       <c r="B125" t="s">
+        <v>34</v>
+      </c>
+      <c r="C125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>12</v>
+      </c>
+      <c r="B126" t="s">
+        <v>32</v>
+      </c>
+      <c r="C126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>12</v>
+      </c>
+      <c r="B127" t="s">
+        <v>58</v>
+      </c>
+      <c r="C127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>12</v>
+      </c>
+      <c r="B128" t="s">
+        <v>71</v>
+      </c>
+      <c r="C128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>12</v>
+      </c>
+      <c r="B129" t="s">
+        <v>53</v>
+      </c>
+      <c r="C129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>12</v>
+      </c>
+      <c r="B130" t="s">
+        <v>74</v>
+      </c>
+      <c r="C130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>12</v>
+      </c>
+      <c r="B131" t="s">
+        <v>36</v>
+      </c>
+      <c r="C131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>12</v>
+      </c>
+      <c r="B132" t="s">
+        <v>48</v>
+      </c>
+      <c r="C132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>12</v>
+      </c>
+      <c r="B133" t="s">
+        <v>78</v>
+      </c>
+      <c r="C133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>12</v>
+      </c>
+      <c r="B134" t="s">
+        <v>55</v>
+      </c>
+      <c r="C134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>12</v>
+      </c>
+      <c r="B135" t="s">
+        <v>45</v>
+      </c>
+      <c r="C135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
+        <v>12</v>
+      </c>
+      <c r="B136" t="s">
+        <v>75</v>
+      </c>
+      <c r="C136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>12</v>
+      </c>
+      <c r="B137" t="s">
+        <v>76</v>
+      </c>
+      <c r="C137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>12</v>
+      </c>
+      <c r="B138" t="s">
+        <v>78</v>
+      </c>
+      <c r="C138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>11</v>
+      </c>
+      <c r="B139" t="s">
+        <v>69</v>
+      </c>
+      <c r="C139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>12</v>
+      </c>
+      <c r="B140" t="s">
+        <v>69</v>
+      </c>
+      <c r="C140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>12</v>
+      </c>
+      <c r="B141" t="s">
         <v>73</v>
       </c>
-      <c r="C125">
+      <c r="C141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>12</v>
+      </c>
+      <c r="B142" t="s">
+        <v>82</v>
+      </c>
+      <c r="C142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>12</v>
+      </c>
+      <c r="B143" t="s">
+        <v>83</v>
+      </c>
+      <c r="C143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>12</v>
+      </c>
+      <c r="B144" t="s">
+        <v>85</v>
+      </c>
+      <c r="C144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>12</v>
+      </c>
+      <c r="B145" t="s">
+        <v>86</v>
+      </c>
+      <c r="C145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>12</v>
+      </c>
+      <c r="B146" t="s">
+        <v>87</v>
+      </c>
+      <c r="C146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>12</v>
+      </c>
+      <c r="B147" t="s">
+        <v>88</v>
+      </c>
+      <c r="C147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>12</v>
+      </c>
+      <c r="B148" t="s">
+        <v>89</v>
+      </c>
+      <c r="C148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>12</v>
+      </c>
+      <c r="B149" t="s">
+        <v>90</v>
+      </c>
+      <c r="C149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>12</v>
+      </c>
+      <c r="B150" t="s">
+        <v>91</v>
+      </c>
+      <c r="C150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>12</v>
+      </c>
+      <c r="B151" t="s">
+        <v>92</v>
+      </c>
+      <c r="C151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>12</v>
+      </c>
+      <c r="B152" t="s">
+        <v>93</v>
+      </c>
+      <c r="C152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>12</v>
+      </c>
+      <c r="B153" t="s">
+        <v>94</v>
+      </c>
+      <c r="C153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>12</v>
+      </c>
+      <c r="B154" t="s">
+        <v>95</v>
+      </c>
+      <c r="C154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>12</v>
+      </c>
+      <c r="B155" t="s">
+        <v>96</v>
+      </c>
+      <c r="C155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>12</v>
+      </c>
+      <c r="B156" t="s">
+        <v>97</v>
+      </c>
+      <c r="C156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>12</v>
+      </c>
+      <c r="B157" t="s">
+        <v>98</v>
+      </c>
+      <c r="C157">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update TAP capacity data
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6584178-130D-4F54-9B44-93BAE78B7206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D090723C-22A6-4BFE-BF9A-F2325F44EED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1637" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1645" uniqueCount="99">
   <si>
     <t>Commodities</t>
   </si>
@@ -1119,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B154"/>
+  <dimension ref="A1:B155"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2352,6 +2352,14 @@
       </c>
       <c r="B154" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>84</v>
+      </c>
+      <c r="B155" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2361,7 +2369,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I307"/>
+  <dimension ref="A1:I309"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -6119,7 +6127,7 @@
         <v>486.91</v>
       </c>
       <c r="E130">
-        <v>118.77099999999999</v>
+        <v>486.91</v>
       </c>
       <c r="F130">
         <v>1</v>
@@ -6148,7 +6156,7 @@
         <v>144.17500000000001</v>
       </c>
       <c r="E131">
-        <v>118.77099999999999</v>
+        <v>144.17500000000001</v>
       </c>
       <c r="F131">
         <v>1</v>
@@ -6177,7 +6185,7 @@
         <v>49.494</v>
       </c>
       <c r="E132">
-        <v>500</v>
+        <v>49.494</v>
       </c>
       <c r="F132">
         <v>1</v>
@@ -6206,7 +6214,7 @@
         <v>816.06700000000012</v>
       </c>
       <c r="E133">
-        <v>500</v>
+        <v>816.06700000000012</v>
       </c>
       <c r="F133">
         <v>1</v>
@@ -6235,7 +6243,7 @@
         <v>188.88749999999999</v>
       </c>
       <c r="E134">
-        <v>500</v>
+        <v>188.88749999999999</v>
       </c>
       <c r="F134">
         <v>1</v>
@@ -6264,7 +6272,7 @@
         <v>89.716999999999999</v>
       </c>
       <c r="E135">
-        <v>500</v>
+        <v>89.716999999999999</v>
       </c>
       <c r="F135">
         <v>1</v>
@@ -6293,7 +6301,7 @@
         <v>170.63749999999999</v>
       </c>
       <c r="E136">
-        <v>500</v>
+        <v>170.63749999999999</v>
       </c>
       <c r="F136">
         <v>1</v>
@@ -6322,7 +6330,7 @@
         <v>12.1837</v>
       </c>
       <c r="E137">
-        <v>500</v>
+        <v>12.1837</v>
       </c>
       <c r="F137">
         <v>1</v>
@@ -6351,7 +6359,7 @@
         <v>256.15699999999998</v>
       </c>
       <c r="E138">
-        <v>500</v>
+        <v>256.15699999999998</v>
       </c>
       <c r="F138">
         <v>1</v>
@@ -6380,7 +6388,7 @@
         <v>61.32</v>
       </c>
       <c r="E139">
-        <v>500</v>
+        <v>61.32</v>
       </c>
       <c r="F139">
         <v>1</v>
@@ -6409,7 +6417,7 @@
         <v>180.20050000000001</v>
       </c>
       <c r="E140">
-        <v>500</v>
+        <v>180.20050000000001</v>
       </c>
       <c r="F140">
         <v>1</v>
@@ -6438,7 +6446,7 @@
         <v>421.21</v>
       </c>
       <c r="E141">
-        <v>500</v>
+        <v>421.21</v>
       </c>
       <c r="F141">
         <v>1</v>
@@ -6467,7 +6475,7 @@
         <v>123.04150000000001</v>
       </c>
       <c r="E142">
-        <v>500</v>
+        <v>123.04150000000001</v>
       </c>
       <c r="F142">
         <v>1</v>
@@ -6496,7 +6504,7 @@
         <v>161.62200000000001</v>
       </c>
       <c r="E143">
-        <v>500</v>
+        <v>161.62200000000001</v>
       </c>
       <c r="F143">
         <v>1</v>
@@ -6525,7 +6533,7 @@
         <v>455.15499999999997</v>
       </c>
       <c r="E144">
-        <v>500</v>
+        <v>455.15499999999997</v>
       </c>
       <c r="F144">
         <v>1</v>
@@ -6554,7 +6562,7 @@
         <v>351.714</v>
       </c>
       <c r="E145">
-        <v>500</v>
+        <v>351.714</v>
       </c>
       <c r="F145">
         <v>1</v>
@@ -6583,7 +6591,7 @@
         <v>167.75399999999999</v>
       </c>
       <c r="E146">
-        <v>500</v>
+        <v>167.75399999999999</v>
       </c>
       <c r="F146">
         <v>1</v>
@@ -6612,7 +6620,7 @@
         <v>207.5025</v>
       </c>
       <c r="E147">
-        <v>500</v>
+        <v>207.5025</v>
       </c>
       <c r="F147">
         <v>1</v>
@@ -6641,7 +6649,7 @@
         <v>513.19000000000005</v>
       </c>
       <c r="E148">
-        <v>500</v>
+        <v>513.19000000000005</v>
       </c>
       <c r="F148">
         <v>1</v>
@@ -6670,7 +6678,7 @@
         <v>140.52500000000001</v>
       </c>
       <c r="E149">
-        <v>500</v>
+        <v>140.52500000000001</v>
       </c>
       <c r="F149">
         <v>1</v>
@@ -6699,7 +6707,7 @@
         <v>82.927999999999997</v>
       </c>
       <c r="E150">
-        <v>500</v>
+        <v>82.927999999999997</v>
       </c>
       <c r="F150">
         <v>1</v>
@@ -6728,7 +6736,7 @@
         <v>67.451999999999998</v>
       </c>
       <c r="E151">
-        <v>500</v>
+        <v>67.451999999999998</v>
       </c>
       <c r="F151">
         <v>1</v>
@@ -6754,10 +6762,10 @@
         <v>22</v>
       </c>
       <c r="D152">
-        <v>395</v>
+        <v>200.71350000000001</v>
       </c>
       <c r="E152">
-        <v>395</v>
+        <v>200.71350000000001</v>
       </c>
       <c r="F152">
         <v>1</v>
@@ -6783,10 +6791,10 @@
         <v>74</v>
       </c>
       <c r="D153">
-        <v>395</v>
+        <v>200.71350000000001</v>
       </c>
       <c r="E153">
-        <v>395</v>
+        <v>200.71350000000001</v>
       </c>
       <c r="F153">
         <v>1</v>
@@ -6812,10 +6820,10 @@
         <v>20</v>
       </c>
       <c r="D154">
-        <v>395</v>
+        <v>144.17500000000001</v>
       </c>
       <c r="E154">
-        <v>395</v>
+        <v>144.17500000000001</v>
       </c>
       <c r="F154">
         <v>1</v>
@@ -6832,19 +6840,19 @@
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B155" t="s">
-        <v>15</v>
+        <v>84</v>
       </c>
       <c r="C155" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="D155">
-        <v>500</v>
+        <v>123.04150000000001</v>
       </c>
       <c r="E155">
-        <v>500</v>
+        <v>123.04150000000001</v>
       </c>
       <c r="F155">
         <v>1</v>
@@ -6853,7 +6861,7 @@
         <v>10000000</v>
       </c>
       <c r="H155">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I155">
         <v>1</v>
@@ -6864,10 +6872,10 @@
         <v>12</v>
       </c>
       <c r="B156" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C156" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D156">
         <v>500</v>
@@ -6893,10 +6901,10 @@
         <v>12</v>
       </c>
       <c r="B157" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C157" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D157">
         <v>500</v>
@@ -6922,10 +6930,10 @@
         <v>12</v>
       </c>
       <c r="B158" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C158" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D158">
         <v>500</v>
@@ -6951,10 +6959,10 @@
         <v>12</v>
       </c>
       <c r="B159" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C159" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D159">
         <v>500</v>
@@ -6980,10 +6988,10 @@
         <v>12</v>
       </c>
       <c r="B160" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C160" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D160">
         <v>500</v>
@@ -7009,10 +7017,10 @@
         <v>12</v>
       </c>
       <c r="B161" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C161" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D161">
         <v>500</v>
@@ -7038,10 +7046,10 @@
         <v>12</v>
       </c>
       <c r="B162" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C162" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D162">
         <v>500</v>
@@ -7067,10 +7075,10 @@
         <v>12</v>
       </c>
       <c r="B163" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C163" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D163">
         <v>500</v>
@@ -7096,10 +7104,10 @@
         <v>12</v>
       </c>
       <c r="B164" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C164" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D164">
         <v>500</v>
@@ -7125,10 +7133,10 @@
         <v>12</v>
       </c>
       <c r="B165" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C165" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D165">
         <v>500</v>
@@ -7154,10 +7162,10 @@
         <v>12</v>
       </c>
       <c r="B166" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C166" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D166">
         <v>500</v>
@@ -7183,10 +7191,10 @@
         <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="C167" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="D167">
         <v>500</v>
@@ -7212,10 +7220,10 @@
         <v>12</v>
       </c>
       <c r="B168" t="s">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C168" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="D168">
         <v>500</v>
@@ -7241,10 +7249,10 @@
         <v>12</v>
       </c>
       <c r="B169" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D169">
         <v>500</v>
@@ -7270,10 +7278,10 @@
         <v>12</v>
       </c>
       <c r="B170" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C170" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D170">
         <v>500</v>
@@ -7299,10 +7307,10 @@
         <v>12</v>
       </c>
       <c r="B171" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C171" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D171">
         <v>500</v>
@@ -7328,10 +7336,10 @@
         <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C172" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D172">
         <v>500</v>
@@ -7357,10 +7365,10 @@
         <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C173" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="D173">
         <v>500</v>
@@ -7386,10 +7394,10 @@
         <v>12</v>
       </c>
       <c r="B174" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C174" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="D174">
         <v>500</v>
@@ -7415,10 +7423,10 @@
         <v>12</v>
       </c>
       <c r="B175" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C175" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="D175">
         <v>500</v>
@@ -7444,10 +7452,10 @@
         <v>12</v>
       </c>
       <c r="B176" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C176" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D176">
         <v>500</v>
@@ -7473,10 +7481,10 @@
         <v>12</v>
       </c>
       <c r="B177" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C177" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D177">
         <v>500</v>
@@ -7502,10 +7510,10 @@
         <v>12</v>
       </c>
       <c r="B178" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C178" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="D178">
         <v>500</v>
@@ -7531,10 +7539,10 @@
         <v>12</v>
       </c>
       <c r="B179" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C179" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="D179">
         <v>500</v>
@@ -7560,10 +7568,10 @@
         <v>12</v>
       </c>
       <c r="B180" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C180" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="D180">
         <v>500</v>
@@ -7592,7 +7600,7 @@
         <v>38</v>
       </c>
       <c r="C181" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="D181">
         <v>500</v>
@@ -7618,10 +7626,10 @@
         <v>12</v>
       </c>
       <c r="B182" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C182" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="D182">
         <v>500</v>
@@ -7650,7 +7658,7 @@
         <v>16</v>
       </c>
       <c r="C183" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D183">
         <v>500</v>
@@ -7679,7 +7687,7 @@
         <v>16</v>
       </c>
       <c r="C184" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D184">
         <v>500</v>
@@ -7708,7 +7716,7 @@
         <v>16</v>
       </c>
       <c r="C185" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D185">
         <v>500</v>
@@ -7734,10 +7742,10 @@
         <v>12</v>
       </c>
       <c r="B186" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C186" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D186">
         <v>500</v>
@@ -7766,7 +7774,7 @@
         <v>28</v>
       </c>
       <c r="C187" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D187">
         <v>500</v>
@@ -7792,10 +7800,10 @@
         <v>12</v>
       </c>
       <c r="B188" t="s">
+        <v>28</v>
+      </c>
+      <c r="C188" t="s">
         <v>42</v>
-      </c>
-      <c r="C188" t="s">
-        <v>16</v>
       </c>
       <c r="D188">
         <v>500</v>
@@ -7824,7 +7832,7 @@
         <v>42</v>
       </c>
       <c r="C189" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D189">
         <v>500</v>
@@ -7853,7 +7861,7 @@
         <v>42</v>
       </c>
       <c r="C190" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="D190">
         <v>500</v>
@@ -7882,7 +7890,7 @@
         <v>42</v>
       </c>
       <c r="C191" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D191">
         <v>500</v>
@@ -7911,7 +7919,7 @@
         <v>42</v>
       </c>
       <c r="C192" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="D192">
         <v>500</v>
@@ -7940,7 +7948,7 @@
         <v>42</v>
       </c>
       <c r="C193" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="D193">
         <v>500</v>
@@ -7969,7 +7977,7 @@
         <v>42</v>
       </c>
       <c r="C194" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D194">
         <v>500</v>
@@ -7998,7 +8006,7 @@
         <v>42</v>
       </c>
       <c r="C195" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="D195">
         <v>500</v>
@@ -8027,7 +8035,7 @@
         <v>42</v>
       </c>
       <c r="C196" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D196">
         <v>500</v>
@@ -8053,10 +8061,10 @@
         <v>12</v>
       </c>
       <c r="B197" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C197" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D197">
         <v>500</v>
@@ -8085,7 +8093,7 @@
         <v>60</v>
       </c>
       <c r="C198" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D198">
         <v>500</v>
@@ -8114,7 +8122,7 @@
         <v>60</v>
       </c>
       <c r="C199" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D199">
         <v>500</v>
@@ -8143,7 +8151,7 @@
         <v>60</v>
       </c>
       <c r="C200" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D200">
         <v>500</v>
@@ -8172,7 +8180,7 @@
         <v>60</v>
       </c>
       <c r="C201" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D201">
         <v>500</v>
@@ -8198,10 +8206,10 @@
         <v>12</v>
       </c>
       <c r="B202" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C202" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D202">
         <v>500</v>
@@ -8230,7 +8238,7 @@
         <v>22</v>
       </c>
       <c r="C203" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D203">
         <v>500</v>
@@ -8259,7 +8267,7 @@
         <v>22</v>
       </c>
       <c r="C204" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D204">
         <v>500</v>
@@ -8285,10 +8293,10 @@
         <v>12</v>
       </c>
       <c r="B205" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="C205" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="D205">
         <v>500</v>
@@ -8317,7 +8325,7 @@
         <v>61</v>
       </c>
       <c r="C206" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D206">
         <v>500</v>
@@ -8346,7 +8354,7 @@
         <v>61</v>
       </c>
       <c r="C207" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D207">
         <v>500</v>
@@ -8372,10 +8380,10 @@
         <v>12</v>
       </c>
       <c r="B208" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C208" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D208">
         <v>500</v>
@@ -8404,7 +8412,7 @@
         <v>64</v>
       </c>
       <c r="C209" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D209">
         <v>500</v>
@@ -8430,10 +8438,10 @@
         <v>12</v>
       </c>
       <c r="B210" t="s">
+        <v>64</v>
+      </c>
+      <c r="C210" t="s">
         <v>24</v>
-      </c>
-      <c r="C210" t="s">
-        <v>64</v>
       </c>
       <c r="D210">
         <v>500</v>
@@ -8462,7 +8470,7 @@
         <v>24</v>
       </c>
       <c r="C211" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D211">
         <v>500</v>
@@ -8488,10 +8496,10 @@
         <v>12</v>
       </c>
       <c r="B212" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C212" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="D212">
         <v>500</v>
@@ -8520,7 +8528,7 @@
         <v>18</v>
       </c>
       <c r="C213" t="s">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="D213">
         <v>500</v>
@@ -8549,7 +8557,7 @@
         <v>18</v>
       </c>
       <c r="C214" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="D214">
         <v>500</v>
@@ -8575,10 +8583,10 @@
         <v>12</v>
       </c>
       <c r="B215" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C215" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D215">
         <v>500</v>
@@ -8604,7 +8612,7 @@
         <v>12</v>
       </c>
       <c r="B216" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C216" t="s">
         <v>42</v>
@@ -8633,7 +8641,7 @@
         <v>12</v>
       </c>
       <c r="B217" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C217" t="s">
         <v>42</v>
@@ -8665,7 +8673,7 @@
         <v>62</v>
       </c>
       <c r="C218" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D218">
         <v>500</v>
@@ -8694,7 +8702,7 @@
         <v>62</v>
       </c>
       <c r="C219" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D219">
         <v>500</v>
@@ -8720,10 +8728,10 @@
         <v>12</v>
       </c>
       <c r="B220" t="s">
+        <v>62</v>
+      </c>
+      <c r="C220" t="s">
         <v>65</v>
-      </c>
-      <c r="C220" t="s">
-        <v>60</v>
       </c>
       <c r="D220">
         <v>500</v>
@@ -8752,7 +8760,7 @@
         <v>65</v>
       </c>
       <c r="C221" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D221">
         <v>500</v>
@@ -8781,7 +8789,7 @@
         <v>65</v>
       </c>
       <c r="C222" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D222">
         <v>500</v>
@@ -8810,7 +8818,7 @@
         <v>65</v>
       </c>
       <c r="C223" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D223">
         <v>500</v>
@@ -8836,10 +8844,10 @@
         <v>12</v>
       </c>
       <c r="B224" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C224" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="D224">
         <v>500</v>
@@ -8868,7 +8876,7 @@
         <v>66</v>
       </c>
       <c r="C225" t="s">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="D225">
         <v>500</v>
@@ -8897,7 +8905,7 @@
         <v>66</v>
       </c>
       <c r="C226" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D226">
         <v>500</v>
@@ -8926,7 +8934,7 @@
         <v>66</v>
       </c>
       <c r="C227" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D227">
         <v>500</v>
@@ -8952,10 +8960,10 @@
         <v>12</v>
       </c>
       <c r="B228" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C228" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="D228">
         <v>500</v>
@@ -8984,7 +8992,7 @@
         <v>67</v>
       </c>
       <c r="C229" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D229">
         <v>500</v>
@@ -9010,10 +9018,10 @@
         <v>12</v>
       </c>
       <c r="B230" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C230" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D230">
         <v>500</v>
@@ -9042,7 +9050,7 @@
         <v>68</v>
       </c>
       <c r="C231" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="D231">
         <v>500</v>
@@ -9071,7 +9079,7 @@
         <v>68</v>
       </c>
       <c r="C232" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="D232">
         <v>500</v>
@@ -9100,7 +9108,7 @@
         <v>68</v>
       </c>
       <c r="C233" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="D233">
         <v>500</v>
@@ -9129,7 +9137,7 @@
         <v>68</v>
       </c>
       <c r="C234" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="D234">
         <v>500</v>
@@ -9155,10 +9163,10 @@
         <v>12</v>
       </c>
       <c r="B235" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C235" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="D235">
         <v>500</v>
@@ -9184,10 +9192,10 @@
         <v>12</v>
       </c>
       <c r="B236" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C236" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D236">
         <v>500</v>
@@ -9216,7 +9224,7 @@
         <v>51</v>
       </c>
       <c r="C237" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D237">
         <v>500</v>
@@ -9245,7 +9253,7 @@
         <v>51</v>
       </c>
       <c r="C238" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D238">
         <v>500</v>
@@ -9274,7 +9282,7 @@
         <v>51</v>
       </c>
       <c r="C239" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="D239">
         <v>500</v>
@@ -9300,10 +9308,10 @@
         <v>12</v>
       </c>
       <c r="B240" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="C240" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D240">
         <v>500</v>
@@ -9332,7 +9340,7 @@
         <v>26</v>
       </c>
       <c r="C241" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="D241">
         <v>500</v>
@@ -9358,10 +9366,10 @@
         <v>12</v>
       </c>
       <c r="B242" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="C242" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="D242">
         <v>500</v>
@@ -9390,7 +9398,7 @@
         <v>72</v>
       </c>
       <c r="C243" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="D243">
         <v>500</v>
@@ -9416,10 +9424,10 @@
         <v>12</v>
       </c>
       <c r="B244" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="C244" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D244">
         <v>500</v>
@@ -9448,7 +9456,7 @@
         <v>34</v>
       </c>
       <c r="C245" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D245">
         <v>500</v>
@@ -9474,10 +9482,10 @@
         <v>12</v>
       </c>
       <c r="B246" t="s">
+        <v>34</v>
+      </c>
+      <c r="C246" t="s">
         <v>32</v>
-      </c>
-      <c r="C246" t="s">
-        <v>34</v>
       </c>
       <c r="D246">
         <v>500</v>
@@ -9503,10 +9511,10 @@
         <v>12</v>
       </c>
       <c r="B247" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="C247" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D247">
         <v>500</v>
@@ -9535,7 +9543,7 @@
         <v>58</v>
       </c>
       <c r="C248" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D248">
         <v>500</v>
@@ -9564,7 +9572,7 @@
         <v>58</v>
       </c>
       <c r="C249" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D249">
         <v>500</v>
@@ -9593,7 +9601,7 @@
         <v>58</v>
       </c>
       <c r="C250" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="D250">
         <v>500</v>
@@ -9619,7 +9627,7 @@
         <v>12</v>
       </c>
       <c r="B251" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C251" t="s">
         <v>51</v>
@@ -9648,10 +9656,10 @@
         <v>12</v>
       </c>
       <c r="B252" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="C252" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="D252">
         <v>500</v>
@@ -9680,7 +9688,7 @@
         <v>53</v>
       </c>
       <c r="C253" t="s">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="D253">
         <v>500</v>
@@ -9709,7 +9717,7 @@
         <v>53</v>
       </c>
       <c r="C254" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D254">
         <v>500</v>
@@ -9735,10 +9743,10 @@
         <v>12</v>
       </c>
       <c r="B255" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C255" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="D255">
         <v>500</v>
@@ -9764,10 +9772,10 @@
         <v>12</v>
       </c>
       <c r="B256" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="C256" t="s">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="D256">
         <v>500</v>
@@ -9796,7 +9804,7 @@
         <v>36</v>
       </c>
       <c r="C257" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="D257">
         <v>500</v>
@@ -9822,10 +9830,10 @@
         <v>12</v>
       </c>
       <c r="B258" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C258" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D258">
         <v>500</v>
@@ -9854,7 +9862,7 @@
         <v>48</v>
       </c>
       <c r="C259" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D259">
         <v>500</v>
@@ -9883,7 +9891,7 @@
         <v>48</v>
       </c>
       <c r="C260" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D260">
         <v>500</v>
@@ -9912,7 +9920,7 @@
         <v>48</v>
       </c>
       <c r="C261" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D261">
         <v>500</v>
@@ -9938,10 +9946,10 @@
         <v>12</v>
       </c>
       <c r="B262" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C262" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="D262">
         <v>500</v>
@@ -9967,10 +9975,10 @@
         <v>12</v>
       </c>
       <c r="B263" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C263" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D263">
         <v>500</v>
@@ -9996,7 +10004,7 @@
         <v>12</v>
       </c>
       <c r="B264" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C264" t="s">
         <v>22</v>
@@ -10025,10 +10033,10 @@
         <v>12</v>
       </c>
       <c r="B265" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="C265" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D265">
         <v>500</v>
@@ -10057,7 +10065,7 @@
         <v>75</v>
       </c>
       <c r="C266" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D266">
         <v>500</v>
@@ -10083,10 +10091,10 @@
         <v>12</v>
       </c>
       <c r="B267" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C267" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="D267">
         <v>500</v>
@@ -10112,10 +10120,10 @@
         <v>12</v>
       </c>
       <c r="B268" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="C268" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D268">
         <v>500</v>
@@ -10141,10 +10149,10 @@
         <v>12</v>
       </c>
       <c r="B269" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C269" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D269">
         <v>500</v>
@@ -10173,7 +10181,7 @@
         <v>58</v>
       </c>
       <c r="C270" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D270">
         <v>500</v>
@@ -10202,7 +10210,7 @@
         <v>58</v>
       </c>
       <c r="C271" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D271">
         <v>500</v>
@@ -10228,7 +10236,7 @@
         <v>12</v>
       </c>
       <c r="B272" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C272" t="s">
         <v>66</v>
@@ -10257,10 +10265,10 @@
         <v>12</v>
       </c>
       <c r="B273" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C273" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D273">
         <v>500</v>
@@ -10289,7 +10297,7 @@
         <v>68</v>
       </c>
       <c r="C274" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D274">
         <v>500</v>
@@ -10315,10 +10323,10 @@
         <v>12</v>
       </c>
       <c r="B275" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="C275" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D275">
         <v>500</v>
@@ -10344,10 +10352,10 @@
         <v>12</v>
       </c>
       <c r="B276" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="C276" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D276">
         <v>500</v>
@@ -10373,10 +10381,10 @@
         <v>12</v>
       </c>
       <c r="B277" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C277" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="D277">
         <v>500</v>
@@ -10402,7 +10410,7 @@
         <v>12</v>
       </c>
       <c r="B278" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C278" t="s">
         <v>22</v>
@@ -10431,10 +10439,10 @@
         <v>12</v>
       </c>
       <c r="B279" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="C279" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="D279">
         <v>500</v>
@@ -10460,7 +10468,7 @@
         <v>12</v>
       </c>
       <c r="B280" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C280" t="s">
         <v>34</v>
@@ -10489,10 +10497,10 @@
         <v>12</v>
       </c>
       <c r="B281" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="C281" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D281">
         <v>500</v>
@@ -10521,7 +10529,7 @@
         <v>48</v>
       </c>
       <c r="C282" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D282">
         <v>500</v>
@@ -10550,7 +10558,7 @@
         <v>48</v>
       </c>
       <c r="C283" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D283">
         <v>500</v>
@@ -10579,7 +10587,7 @@
         <v>48</v>
       </c>
       <c r="C284" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D284">
         <v>500</v>
@@ -10608,7 +10616,7 @@
         <v>48</v>
       </c>
       <c r="C285" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D285">
         <v>500</v>
@@ -10634,10 +10642,10 @@
         <v>12</v>
       </c>
       <c r="B286" t="s">
+        <v>48</v>
+      </c>
+      <c r="C286" t="s">
         <v>38</v>
-      </c>
-      <c r="C286" t="s">
-        <v>79</v>
       </c>
       <c r="D286">
         <v>500</v>
@@ -10666,7 +10674,7 @@
         <v>38</v>
       </c>
       <c r="C287" t="s">
-        <v>16</v>
+        <v>79</v>
       </c>
       <c r="D287">
         <v>500</v>
@@ -10695,7 +10703,7 @@
         <v>38</v>
       </c>
       <c r="C288" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D288">
         <v>500</v>
@@ -10721,10 +10729,10 @@
         <v>12</v>
       </c>
       <c r="B289" t="s">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="C289" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D289">
         <v>500</v>
@@ -10750,10 +10758,10 @@
         <v>12</v>
       </c>
       <c r="B290" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="C290" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D290">
         <v>500</v>
@@ -10779,10 +10787,10 @@
         <v>12</v>
       </c>
       <c r="B291" t="s">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="C291" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="D291">
         <v>500</v>
@@ -10808,19 +10816,19 @@
         <v>12</v>
       </c>
       <c r="B292" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C292" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="D292">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E292">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="F292">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G292">
         <v>10000000</v>
@@ -10837,19 +10845,19 @@
         <v>12</v>
       </c>
       <c r="B293" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C293" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D293">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E293">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="F293">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G293">
         <v>10000000</v>
@@ -10866,10 +10874,10 @@
         <v>12</v>
       </c>
       <c r="B294" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C294" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D294">
         <v>10000</v>
@@ -10895,10 +10903,10 @@
         <v>12</v>
       </c>
       <c r="B295" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C295" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="D295">
         <v>10000</v>
@@ -10924,10 +10932,10 @@
         <v>12</v>
       </c>
       <c r="B296" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C296" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D296">
         <v>10000</v>
@@ -10953,10 +10961,10 @@
         <v>12</v>
       </c>
       <c r="B297" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C297" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D297">
         <v>10000</v>
@@ -10982,10 +10990,10 @@
         <v>12</v>
       </c>
       <c r="B298" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C298" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D298">
         <v>10000</v>
@@ -11011,10 +11019,10 @@
         <v>12</v>
       </c>
       <c r="B299" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C299" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D299">
         <v>10000</v>
@@ -11040,10 +11048,10 @@
         <v>12</v>
       </c>
       <c r="B300" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C300" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="D300">
         <v>10000</v>
@@ -11069,10 +11077,10 @@
         <v>12</v>
       </c>
       <c r="B301" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C301" t="s">
-        <v>66</v>
+        <v>18</v>
       </c>
       <c r="D301">
         <v>10000</v>
@@ -11098,10 +11106,10 @@
         <v>12</v>
       </c>
       <c r="B302" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C302" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="D302">
         <v>10000</v>
@@ -11127,10 +11135,10 @@
         <v>12</v>
       </c>
       <c r="B303" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C303" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D303">
         <v>10000</v>
@@ -11156,10 +11164,10 @@
         <v>12</v>
       </c>
       <c r="B304" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C304" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D304">
         <v>10000</v>
@@ -11185,10 +11193,10 @@
         <v>12</v>
       </c>
       <c r="B305" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C305" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D305">
         <v>10000</v>
@@ -11214,10 +11222,10 @@
         <v>12</v>
       </c>
       <c r="B306" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C306" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D306">
         <v>10000</v>
@@ -11243,10 +11251,10 @@
         <v>12</v>
       </c>
       <c r="B307" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C307" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="D307">
         <v>10000</v>
@@ -11264,6 +11272,64 @@
         <v>1000</v>
       </c>
       <c r="I307">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="308" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A308" t="s">
+        <v>12</v>
+      </c>
+      <c r="B308" t="s">
+        <v>97</v>
+      </c>
+      <c r="C308" t="s">
+        <v>36</v>
+      </c>
+      <c r="D308">
+        <v>10000</v>
+      </c>
+      <c r="E308">
+        <v>10000</v>
+      </c>
+      <c r="F308">
+        <v>100</v>
+      </c>
+      <c r="G308">
+        <v>10000000</v>
+      </c>
+      <c r="H308">
+        <v>1000</v>
+      </c>
+      <c r="I308">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A309" t="s">
+        <v>12</v>
+      </c>
+      <c r="B309" t="s">
+        <v>98</v>
+      </c>
+      <c r="C309" t="s">
+        <v>34</v>
+      </c>
+      <c r="D309">
+        <v>10000</v>
+      </c>
+      <c r="E309">
+        <v>10000</v>
+      </c>
+      <c r="F309">
+        <v>100</v>
+      </c>
+      <c r="G309">
+        <v>10000000</v>
+      </c>
+      <c r="H309">
+        <v>1000</v>
+      </c>
+      <c r="I309">
         <v>1</v>
       </c>
     </row>
@@ -11297,7 +11363,7 @@
         <v>15</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>111.378</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -11308,7 +11374,7 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>322.40999999999997</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -11319,7 +11385,7 @@
         <v>19</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>73.274999999999991</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -11330,7 +11396,7 @@
         <v>21</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>155.83149999999998</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -11341,7 +11407,7 @@
         <v>23</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>25.402000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -11352,7 +11418,7 @@
         <v>25</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>39.08</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -11363,7 +11429,7 @@
         <v>27</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>122.125</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -11374,7 +11440,7 @@
         <v>29</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>60.573999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -11385,7 +11451,7 @@
         <v>31</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>74.251999999999995</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -11396,7 +11462,7 @@
         <v>33</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>655.56699999999989</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -11407,7 +11473,7 @@
         <v>35</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>425.97199999999998</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -11418,7 +11484,7 @@
         <v>37</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>510.97099999999995</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
update data for MENA imports
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D090723C-22A6-4BFE-BF9A-F2325F44EED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670EB0CF-6BF9-4B32-A097-98F6C60D675C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1645" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1653" uniqueCount="99">
   <si>
     <t>Commodities</t>
   </si>
@@ -1119,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B155"/>
+  <dimension ref="A1:B156"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2360,6 +2360,14 @@
       </c>
       <c r="B155" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>84</v>
+      </c>
+      <c r="B156" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2369,7 +2377,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I309"/>
+  <dimension ref="A1:I311"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -6869,19 +6877,19 @@
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B156" t="s">
-        <v>15</v>
+        <v>84</v>
       </c>
       <c r="C156" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="D156">
-        <v>500</v>
+        <v>421.21</v>
       </c>
       <c r="E156">
-        <v>500</v>
+        <v>421.21</v>
       </c>
       <c r="F156">
         <v>1</v>
@@ -6890,7 +6898,7 @@
         <v>10000000</v>
       </c>
       <c r="H156">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I156">
         <v>1</v>
@@ -6901,10 +6909,10 @@
         <v>12</v>
       </c>
       <c r="B157" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C157" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D157">
         <v>500</v>
@@ -6930,10 +6938,10 @@
         <v>12</v>
       </c>
       <c r="B158" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C158" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D158">
         <v>500</v>
@@ -6959,10 +6967,10 @@
         <v>12</v>
       </c>
       <c r="B159" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C159" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D159">
         <v>500</v>
@@ -6988,10 +6996,10 @@
         <v>12</v>
       </c>
       <c r="B160" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C160" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D160">
         <v>500</v>
@@ -7017,10 +7025,10 @@
         <v>12</v>
       </c>
       <c r="B161" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C161" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D161">
         <v>500</v>
@@ -7046,10 +7054,10 @@
         <v>12</v>
       </c>
       <c r="B162" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C162" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D162">
         <v>500</v>
@@ -7075,10 +7083,10 @@
         <v>12</v>
       </c>
       <c r="B163" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C163" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D163">
         <v>500</v>
@@ -7104,10 +7112,10 @@
         <v>12</v>
       </c>
       <c r="B164" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C164" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D164">
         <v>500</v>
@@ -7133,10 +7141,10 @@
         <v>12</v>
       </c>
       <c r="B165" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C165" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D165">
         <v>500</v>
@@ -7162,10 +7170,10 @@
         <v>12</v>
       </c>
       <c r="B166" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C166" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D166">
         <v>500</v>
@@ -7191,10 +7199,10 @@
         <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C167" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D167">
         <v>500</v>
@@ -7220,10 +7228,10 @@
         <v>12</v>
       </c>
       <c r="B168" t="s">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="C168" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="D168">
         <v>500</v>
@@ -7249,10 +7257,10 @@
         <v>12</v>
       </c>
       <c r="B169" t="s">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C169" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="D169">
         <v>500</v>
@@ -7278,10 +7286,10 @@
         <v>12</v>
       </c>
       <c r="B170" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D170">
         <v>500</v>
@@ -7307,10 +7315,10 @@
         <v>12</v>
       </c>
       <c r="B171" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C171" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D171">
         <v>500</v>
@@ -7336,10 +7344,10 @@
         <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C172" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D172">
         <v>500</v>
@@ -7365,10 +7373,10 @@
         <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C173" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D173">
         <v>500</v>
@@ -7394,10 +7402,10 @@
         <v>12</v>
       </c>
       <c r="B174" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C174" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="D174">
         <v>500</v>
@@ -7423,10 +7431,10 @@
         <v>12</v>
       </c>
       <c r="B175" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C175" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="D175">
         <v>500</v>
@@ -7452,10 +7460,10 @@
         <v>12</v>
       </c>
       <c r="B176" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C176" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="D176">
         <v>500</v>
@@ -7481,10 +7489,10 @@
         <v>12</v>
       </c>
       <c r="B177" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C177" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D177">
         <v>500</v>
@@ -7510,10 +7518,10 @@
         <v>12</v>
       </c>
       <c r="B178" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C178" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D178">
         <v>500</v>
@@ -7539,10 +7547,10 @@
         <v>12</v>
       </c>
       <c r="B179" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C179" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="D179">
         <v>500</v>
@@ -7568,10 +7576,10 @@
         <v>12</v>
       </c>
       <c r="B180" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C180" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="D180">
         <v>500</v>
@@ -7597,10 +7605,10 @@
         <v>12</v>
       </c>
       <c r="B181" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C181" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="D181">
         <v>500</v>
@@ -7629,7 +7637,7 @@
         <v>38</v>
       </c>
       <c r="C182" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="D182">
         <v>500</v>
@@ -7655,10 +7663,10 @@
         <v>12</v>
       </c>
       <c r="B183" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C183" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="D183">
         <v>500</v>
@@ -7687,7 +7695,7 @@
         <v>16</v>
       </c>
       <c r="C184" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D184">
         <v>500</v>
@@ -7716,7 +7724,7 @@
         <v>16</v>
       </c>
       <c r="C185" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D185">
         <v>500</v>
@@ -7745,7 +7753,7 @@
         <v>16</v>
       </c>
       <c r="C186" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D186">
         <v>500</v>
@@ -7771,10 +7779,10 @@
         <v>12</v>
       </c>
       <c r="B187" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C187" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D187">
         <v>500</v>
@@ -7803,7 +7811,7 @@
         <v>28</v>
       </c>
       <c r="C188" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D188">
         <v>500</v>
@@ -7829,10 +7837,10 @@
         <v>12</v>
       </c>
       <c r="B189" t="s">
+        <v>28</v>
+      </c>
+      <c r="C189" t="s">
         <v>42</v>
-      </c>
-      <c r="C189" t="s">
-        <v>16</v>
       </c>
       <c r="D189">
         <v>500</v>
@@ -7861,7 +7869,7 @@
         <v>42</v>
       </c>
       <c r="C190" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D190">
         <v>500</v>
@@ -7890,7 +7898,7 @@
         <v>42</v>
       </c>
       <c r="C191" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="D191">
         <v>500</v>
@@ -7919,7 +7927,7 @@
         <v>42</v>
       </c>
       <c r="C192" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D192">
         <v>500</v>
@@ -7948,7 +7956,7 @@
         <v>42</v>
       </c>
       <c r="C193" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="D193">
         <v>500</v>
@@ -7977,7 +7985,7 @@
         <v>42</v>
       </c>
       <c r="C194" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="D194">
         <v>500</v>
@@ -8006,7 +8014,7 @@
         <v>42</v>
       </c>
       <c r="C195" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D195">
         <v>500</v>
@@ -8035,7 +8043,7 @@
         <v>42</v>
       </c>
       <c r="C196" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="D196">
         <v>500</v>
@@ -8064,7 +8072,7 @@
         <v>42</v>
       </c>
       <c r="C197" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D197">
         <v>500</v>
@@ -8090,10 +8098,10 @@
         <v>12</v>
       </c>
       <c r="B198" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C198" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D198">
         <v>500</v>
@@ -8122,7 +8130,7 @@
         <v>60</v>
       </c>
       <c r="C199" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D199">
         <v>500</v>
@@ -8151,7 +8159,7 @@
         <v>60</v>
       </c>
       <c r="C200" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D200">
         <v>500</v>
@@ -8180,7 +8188,7 @@
         <v>60</v>
       </c>
       <c r="C201" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D201">
         <v>500</v>
@@ -8209,7 +8217,7 @@
         <v>60</v>
       </c>
       <c r="C202" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D202">
         <v>500</v>
@@ -8235,10 +8243,10 @@
         <v>12</v>
       </c>
       <c r="B203" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C203" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D203">
         <v>500</v>
@@ -8267,7 +8275,7 @@
         <v>22</v>
       </c>
       <c r="C204" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D204">
         <v>500</v>
@@ -8296,7 +8304,7 @@
         <v>22</v>
       </c>
       <c r="C205" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D205">
         <v>500</v>
@@ -8322,10 +8330,10 @@
         <v>12</v>
       </c>
       <c r="B206" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="C206" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="D206">
         <v>500</v>
@@ -8354,7 +8362,7 @@
         <v>61</v>
       </c>
       <c r="C207" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D207">
         <v>500</v>
@@ -8383,7 +8391,7 @@
         <v>61</v>
       </c>
       <c r="C208" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D208">
         <v>500</v>
@@ -8409,10 +8417,10 @@
         <v>12</v>
       </c>
       <c r="B209" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C209" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D209">
         <v>500</v>
@@ -8441,7 +8449,7 @@
         <v>64</v>
       </c>
       <c r="C210" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D210">
         <v>500</v>
@@ -8467,10 +8475,10 @@
         <v>12</v>
       </c>
       <c r="B211" t="s">
+        <v>64</v>
+      </c>
+      <c r="C211" t="s">
         <v>24</v>
-      </c>
-      <c r="C211" t="s">
-        <v>64</v>
       </c>
       <c r="D211">
         <v>500</v>
@@ -8499,7 +8507,7 @@
         <v>24</v>
       </c>
       <c r="C212" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D212">
         <v>500</v>
@@ -8525,10 +8533,10 @@
         <v>12</v>
       </c>
       <c r="B213" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C213" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="D213">
         <v>500</v>
@@ -8557,7 +8565,7 @@
         <v>18</v>
       </c>
       <c r="C214" t="s">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="D214">
         <v>500</v>
@@ -8586,7 +8594,7 @@
         <v>18</v>
       </c>
       <c r="C215" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="D215">
         <v>500</v>
@@ -8612,10 +8620,10 @@
         <v>12</v>
       </c>
       <c r="B216" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C216" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D216">
         <v>500</v>
@@ -8641,7 +8649,7 @@
         <v>12</v>
       </c>
       <c r="B217" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C217" t="s">
         <v>42</v>
@@ -8670,7 +8678,7 @@
         <v>12</v>
       </c>
       <c r="B218" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C218" t="s">
         <v>42</v>
@@ -8702,7 +8710,7 @@
         <v>62</v>
       </c>
       <c r="C219" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D219">
         <v>500</v>
@@ -8731,7 +8739,7 @@
         <v>62</v>
       </c>
       <c r="C220" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D220">
         <v>500</v>
@@ -8757,10 +8765,10 @@
         <v>12</v>
       </c>
       <c r="B221" t="s">
+        <v>62</v>
+      </c>
+      <c r="C221" t="s">
         <v>65</v>
-      </c>
-      <c r="C221" t="s">
-        <v>60</v>
       </c>
       <c r="D221">
         <v>500</v>
@@ -8789,7 +8797,7 @@
         <v>65</v>
       </c>
       <c r="C222" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D222">
         <v>500</v>
@@ -8818,7 +8826,7 @@
         <v>65</v>
       </c>
       <c r="C223" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D223">
         <v>500</v>
@@ -8847,7 +8855,7 @@
         <v>65</v>
       </c>
       <c r="C224" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D224">
         <v>500</v>
@@ -8873,10 +8881,10 @@
         <v>12</v>
       </c>
       <c r="B225" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C225" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="D225">
         <v>500</v>
@@ -8905,7 +8913,7 @@
         <v>66</v>
       </c>
       <c r="C226" t="s">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="D226">
         <v>500</v>
@@ -8934,7 +8942,7 @@
         <v>66</v>
       </c>
       <c r="C227" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D227">
         <v>500</v>
@@ -8963,7 +8971,7 @@
         <v>66</v>
       </c>
       <c r="C228" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D228">
         <v>500</v>
@@ -8989,10 +8997,10 @@
         <v>12</v>
       </c>
       <c r="B229" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C229" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="D229">
         <v>500</v>
@@ -9021,7 +9029,7 @@
         <v>67</v>
       </c>
       <c r="C230" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D230">
         <v>500</v>
@@ -9047,10 +9055,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C231" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D231">
         <v>500</v>
@@ -9079,7 +9087,7 @@
         <v>68</v>
       </c>
       <c r="C232" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="D232">
         <v>500</v>
@@ -9108,7 +9116,7 @@
         <v>68</v>
       </c>
       <c r="C233" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="D233">
         <v>500</v>
@@ -9137,7 +9145,7 @@
         <v>68</v>
       </c>
       <c r="C234" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="D234">
         <v>500</v>
@@ -9166,7 +9174,7 @@
         <v>68</v>
       </c>
       <c r="C235" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="D235">
         <v>500</v>
@@ -9192,10 +9200,10 @@
         <v>12</v>
       </c>
       <c r="B236" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C236" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="D236">
         <v>500</v>
@@ -9221,10 +9229,10 @@
         <v>12</v>
       </c>
       <c r="B237" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C237" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D237">
         <v>500</v>
@@ -9253,7 +9261,7 @@
         <v>51</v>
       </c>
       <c r="C238" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D238">
         <v>500</v>
@@ -9282,7 +9290,7 @@
         <v>51</v>
       </c>
       <c r="C239" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D239">
         <v>500</v>
@@ -9311,7 +9319,7 @@
         <v>51</v>
       </c>
       <c r="C240" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="D240">
         <v>500</v>
@@ -9337,10 +9345,10 @@
         <v>12</v>
       </c>
       <c r="B241" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="C241" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D241">
         <v>500</v>
@@ -9369,7 +9377,7 @@
         <v>26</v>
       </c>
       <c r="C242" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="D242">
         <v>500</v>
@@ -9395,10 +9403,10 @@
         <v>12</v>
       </c>
       <c r="B243" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="C243" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="D243">
         <v>500</v>
@@ -9427,7 +9435,7 @@
         <v>72</v>
       </c>
       <c r="C244" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="D244">
         <v>500</v>
@@ -9453,10 +9461,10 @@
         <v>12</v>
       </c>
       <c r="B245" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="C245" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D245">
         <v>500</v>
@@ -9485,7 +9493,7 @@
         <v>34</v>
       </c>
       <c r="C246" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D246">
         <v>500</v>
@@ -9511,10 +9519,10 @@
         <v>12</v>
       </c>
       <c r="B247" t="s">
+        <v>34</v>
+      </c>
+      <c r="C247" t="s">
         <v>32</v>
-      </c>
-      <c r="C247" t="s">
-        <v>34</v>
       </c>
       <c r="D247">
         <v>500</v>
@@ -9540,10 +9548,10 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="C248" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D248">
         <v>500</v>
@@ -9572,7 +9580,7 @@
         <v>58</v>
       </c>
       <c r="C249" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D249">
         <v>500</v>
@@ -9601,7 +9609,7 @@
         <v>58</v>
       </c>
       <c r="C250" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D250">
         <v>500</v>
@@ -9630,7 +9638,7 @@
         <v>58</v>
       </c>
       <c r="C251" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="D251">
         <v>500</v>
@@ -9656,7 +9664,7 @@
         <v>12</v>
       </c>
       <c r="B252" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C252" t="s">
         <v>51</v>
@@ -9685,10 +9693,10 @@
         <v>12</v>
       </c>
       <c r="B253" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="C253" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="D253">
         <v>500</v>
@@ -9717,7 +9725,7 @@
         <v>53</v>
       </c>
       <c r="C254" t="s">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="D254">
         <v>500</v>
@@ -9746,7 +9754,7 @@
         <v>53</v>
       </c>
       <c r="C255" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D255">
         <v>500</v>
@@ -9772,10 +9780,10 @@
         <v>12</v>
       </c>
       <c r="B256" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C256" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="D256">
         <v>500</v>
@@ -9801,10 +9809,10 @@
         <v>12</v>
       </c>
       <c r="B257" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="C257" t="s">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="D257">
         <v>500</v>
@@ -9833,7 +9841,7 @@
         <v>36</v>
       </c>
       <c r="C258" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="D258">
         <v>500</v>
@@ -9859,10 +9867,10 @@
         <v>12</v>
       </c>
       <c r="B259" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C259" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D259">
         <v>500</v>
@@ -9891,7 +9899,7 @@
         <v>48</v>
       </c>
       <c r="C260" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D260">
         <v>500</v>
@@ -9920,7 +9928,7 @@
         <v>48</v>
       </c>
       <c r="C261" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D261">
         <v>500</v>
@@ -9949,7 +9957,7 @@
         <v>48</v>
       </c>
       <c r="C262" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D262">
         <v>500</v>
@@ -9975,10 +9983,10 @@
         <v>12</v>
       </c>
       <c r="B263" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C263" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="D263">
         <v>500</v>
@@ -10004,10 +10012,10 @@
         <v>12</v>
       </c>
       <c r="B264" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C264" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D264">
         <v>500</v>
@@ -10033,7 +10041,7 @@
         <v>12</v>
       </c>
       <c r="B265" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C265" t="s">
         <v>22</v>
@@ -10062,10 +10070,10 @@
         <v>12</v>
       </c>
       <c r="B266" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="C266" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D266">
         <v>500</v>
@@ -10094,7 +10102,7 @@
         <v>75</v>
       </c>
       <c r="C267" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D267">
         <v>500</v>
@@ -10120,10 +10128,10 @@
         <v>12</v>
       </c>
       <c r="B268" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C268" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="D268">
         <v>500</v>
@@ -10149,10 +10157,10 @@
         <v>12</v>
       </c>
       <c r="B269" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="C269" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D269">
         <v>500</v>
@@ -10178,10 +10186,10 @@
         <v>12</v>
       </c>
       <c r="B270" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C270" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D270">
         <v>500</v>
@@ -10210,7 +10218,7 @@
         <v>58</v>
       </c>
       <c r="C271" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D271">
         <v>500</v>
@@ -10239,7 +10247,7 @@
         <v>58</v>
       </c>
       <c r="C272" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D272">
         <v>500</v>
@@ -10265,7 +10273,7 @@
         <v>12</v>
       </c>
       <c r="B273" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C273" t="s">
         <v>66</v>
@@ -10294,10 +10302,10 @@
         <v>12</v>
       </c>
       <c r="B274" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C274" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D274">
         <v>500</v>
@@ -10326,7 +10334,7 @@
         <v>68</v>
       </c>
       <c r="C275" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D275">
         <v>500</v>
@@ -10352,10 +10360,10 @@
         <v>12</v>
       </c>
       <c r="B276" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="C276" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D276">
         <v>500</v>
@@ -10381,10 +10389,10 @@
         <v>12</v>
       </c>
       <c r="B277" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="C277" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D277">
         <v>500</v>
@@ -10410,10 +10418,10 @@
         <v>12</v>
       </c>
       <c r="B278" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C278" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="D278">
         <v>500</v>
@@ -10439,7 +10447,7 @@
         <v>12</v>
       </c>
       <c r="B279" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C279" t="s">
         <v>22</v>
@@ -10468,10 +10476,10 @@
         <v>12</v>
       </c>
       <c r="B280" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="C280" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="D280">
         <v>500</v>
@@ -10497,7 +10505,7 @@
         <v>12</v>
       </c>
       <c r="B281" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C281" t="s">
         <v>34</v>
@@ -10526,10 +10534,10 @@
         <v>12</v>
       </c>
       <c r="B282" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="C282" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D282">
         <v>500</v>
@@ -10558,7 +10566,7 @@
         <v>48</v>
       </c>
       <c r="C283" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D283">
         <v>500</v>
@@ -10587,7 +10595,7 @@
         <v>48</v>
       </c>
       <c r="C284" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D284">
         <v>500</v>
@@ -10616,7 +10624,7 @@
         <v>48</v>
       </c>
       <c r="C285" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D285">
         <v>500</v>
@@ -10645,7 +10653,7 @@
         <v>48</v>
       </c>
       <c r="C286" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D286">
         <v>500</v>
@@ -10671,10 +10679,10 @@
         <v>12</v>
       </c>
       <c r="B287" t="s">
+        <v>48</v>
+      </c>
+      <c r="C287" t="s">
         <v>38</v>
-      </c>
-      <c r="C287" t="s">
-        <v>79</v>
       </c>
       <c r="D287">
         <v>500</v>
@@ -10703,7 +10711,7 @@
         <v>38</v>
       </c>
       <c r="C288" t="s">
-        <v>16</v>
+        <v>79</v>
       </c>
       <c r="D288">
         <v>500</v>
@@ -10732,7 +10740,7 @@
         <v>38</v>
       </c>
       <c r="C289" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D289">
         <v>500</v>
@@ -10758,10 +10766,10 @@
         <v>12</v>
       </c>
       <c r="B290" t="s">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="C290" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D290">
         <v>500</v>
@@ -10787,10 +10795,10 @@
         <v>12</v>
       </c>
       <c r="B291" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="C291" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D291">
         <v>500</v>
@@ -10816,10 +10824,10 @@
         <v>12</v>
       </c>
       <c r="B292" t="s">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="C292" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="D292">
         <v>500</v>
@@ -10845,10 +10853,10 @@
         <v>12</v>
       </c>
       <c r="B293" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C293" t="s">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="D293">
         <v>500</v>
@@ -10874,19 +10882,19 @@
         <v>12</v>
       </c>
       <c r="B294" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C294" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D294">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E294">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="F294">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G294">
         <v>10000000</v>
@@ -10900,22 +10908,22 @@
     </row>
     <row r="295" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B295" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C295" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="D295">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E295">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="F295">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G295">
         <v>10000000</v>
@@ -10932,10 +10940,10 @@
         <v>12</v>
       </c>
       <c r="B296" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C296" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D296">
         <v>10000</v>
@@ -10961,10 +10969,10 @@
         <v>12</v>
       </c>
       <c r="B297" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C297" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="D297">
         <v>10000</v>
@@ -10990,10 +10998,10 @@
         <v>12</v>
       </c>
       <c r="B298" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C298" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D298">
         <v>10000</v>
@@ -11019,10 +11027,10 @@
         <v>12</v>
       </c>
       <c r="B299" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C299" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D299">
         <v>10000</v>
@@ -11048,10 +11056,10 @@
         <v>12</v>
       </c>
       <c r="B300" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C300" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D300">
         <v>10000</v>
@@ -11077,10 +11085,10 @@
         <v>12</v>
       </c>
       <c r="B301" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C301" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D301">
         <v>10000</v>
@@ -11106,10 +11114,10 @@
         <v>12</v>
       </c>
       <c r="B302" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C302" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="D302">
         <v>10000</v>
@@ -11135,10 +11143,10 @@
         <v>12</v>
       </c>
       <c r="B303" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C303" t="s">
-        <v>66</v>
+        <v>18</v>
       </c>
       <c r="D303">
         <v>10000</v>
@@ -11164,10 +11172,10 @@
         <v>12</v>
       </c>
       <c r="B304" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C304" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="D304">
         <v>10000</v>
@@ -11193,10 +11201,10 @@
         <v>12</v>
       </c>
       <c r="B305" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C305" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D305">
         <v>10000</v>
@@ -11222,10 +11230,10 @@
         <v>12</v>
       </c>
       <c r="B306" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C306" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D306">
         <v>10000</v>
@@ -11251,10 +11259,10 @@
         <v>12</v>
       </c>
       <c r="B307" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C307" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D307">
         <v>10000</v>
@@ -11280,10 +11288,10 @@
         <v>12</v>
       </c>
       <c r="B308" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C308" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D308">
         <v>10000</v>
@@ -11309,10 +11317,10 @@
         <v>12</v>
       </c>
       <c r="B309" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C309" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="D309">
         <v>10000</v>
@@ -11330,6 +11338,64 @@
         <v>1000</v>
       </c>
       <c r="I309">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A310" t="s">
+        <v>12</v>
+      </c>
+      <c r="B310" t="s">
+        <v>97</v>
+      </c>
+      <c r="C310" t="s">
+        <v>36</v>
+      </c>
+      <c r="D310">
+        <v>10000</v>
+      </c>
+      <c r="E310">
+        <v>10000</v>
+      </c>
+      <c r="F310">
+        <v>100</v>
+      </c>
+      <c r="G310">
+        <v>10000000</v>
+      </c>
+      <c r="H310">
+        <v>1000</v>
+      </c>
+      <c r="I310">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A311" t="s">
+        <v>12</v>
+      </c>
+      <c r="B311" t="s">
+        <v>98</v>
+      </c>
+      <c r="C311" t="s">
+        <v>34</v>
+      </c>
+      <c r="D311">
+        <v>10000</v>
+      </c>
+      <c r="E311">
+        <v>10000</v>
+      </c>
+      <c r="F311">
+        <v>100</v>
+      </c>
+      <c r="G311">
+        <v>10000000</v>
+      </c>
+      <c r="H311">
+        <v>1000</v>
+      </c>
+      <c r="I311">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adjust demands per node
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670EB0CF-6BF9-4B32-A097-98F6C60D675C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640808F7-3D5D-4B0C-932E-02E9AB3AEDB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1653" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="99">
   <si>
     <t>Commodities</t>
   </si>
@@ -694,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B0CB446-BDDD-415D-AF22-2CEB1FE45CA5}">
-  <dimension ref="A1:A78"/>
+  <dimension ref="A1:A79"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -1085,6 +1085,11 @@
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>98</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B156"/>
+  <dimension ref="A1:B157"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2368,6 +2373,14 @@
       </c>
       <c r="B156" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>40</v>
+      </c>
+      <c r="B157" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2377,7 +2390,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I311"/>
+  <dimension ref="A1:I313"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -5320,10 +5333,10 @@
         <v>71</v>
       </c>
       <c r="D102">
-        <v>5.8765000000000009</v>
+        <v>20.330500000000001</v>
       </c>
       <c r="E102">
-        <v>5.8765000000000009</v>
+        <v>20.330500000000001</v>
       </c>
       <c r="F102">
         <v>1</v>
@@ -6906,19 +6919,19 @@
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B157" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C157" t="s">
-        <v>16</v>
+        <v>81</v>
       </c>
       <c r="D157">
-        <v>500</v>
+        <v>14.965</v>
       </c>
       <c r="E157">
-        <v>500</v>
+        <v>14.965</v>
       </c>
       <c r="F157">
         <v>1</v>
@@ -6927,7 +6940,7 @@
         <v>10000000</v>
       </c>
       <c r="H157">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I157">
         <v>1</v>
@@ -6938,10 +6951,10 @@
         <v>12</v>
       </c>
       <c r="B158" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C158" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D158">
         <v>500</v>
@@ -6967,10 +6980,10 @@
         <v>12</v>
       </c>
       <c r="B159" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C159" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D159">
         <v>500</v>
@@ -6996,10 +7009,10 @@
         <v>12</v>
       </c>
       <c r="B160" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C160" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D160">
         <v>500</v>
@@ -7025,10 +7038,10 @@
         <v>12</v>
       </c>
       <c r="B161" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C161" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D161">
         <v>500</v>
@@ -7054,10 +7067,10 @@
         <v>12</v>
       </c>
       <c r="B162" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C162" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D162">
         <v>500</v>
@@ -7083,10 +7096,10 @@
         <v>12</v>
       </c>
       <c r="B163" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C163" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D163">
         <v>500</v>
@@ -7112,10 +7125,10 @@
         <v>12</v>
       </c>
       <c r="B164" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C164" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D164">
         <v>500</v>
@@ -7141,10 +7154,10 @@
         <v>12</v>
       </c>
       <c r="B165" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C165" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D165">
         <v>500</v>
@@ -7170,10 +7183,10 @@
         <v>12</v>
       </c>
       <c r="B166" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C166" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D166">
         <v>500</v>
@@ -7199,10 +7212,10 @@
         <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C167" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D167">
         <v>500</v>
@@ -7228,10 +7241,10 @@
         <v>12</v>
       </c>
       <c r="B168" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C168" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D168">
         <v>500</v>
@@ -7257,10 +7270,10 @@
         <v>12</v>
       </c>
       <c r="B169" t="s">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="C169" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="D169">
         <v>500</v>
@@ -7286,10 +7299,10 @@
         <v>12</v>
       </c>
       <c r="B170" t="s">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C170" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="D170">
         <v>500</v>
@@ -7315,10 +7328,10 @@
         <v>12</v>
       </c>
       <c r="B171" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C171" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D171">
         <v>500</v>
@@ -7344,10 +7357,10 @@
         <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C172" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D172">
         <v>500</v>
@@ -7373,10 +7386,10 @@
         <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C173" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D173">
         <v>500</v>
@@ -7402,10 +7415,10 @@
         <v>12</v>
       </c>
       <c r="B174" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C174" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D174">
         <v>500</v>
@@ -7431,10 +7444,10 @@
         <v>12</v>
       </c>
       <c r="B175" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C175" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="D175">
         <v>500</v>
@@ -7460,10 +7473,10 @@
         <v>12</v>
       </c>
       <c r="B176" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C176" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="D176">
         <v>500</v>
@@ -7489,10 +7502,10 @@
         <v>12</v>
       </c>
       <c r="B177" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C177" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="D177">
         <v>500</v>
@@ -7518,10 +7531,10 @@
         <v>12</v>
       </c>
       <c r="B178" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C178" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D178">
         <v>500</v>
@@ -7547,10 +7560,10 @@
         <v>12</v>
       </c>
       <c r="B179" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C179" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D179">
         <v>500</v>
@@ -7576,10 +7589,10 @@
         <v>12</v>
       </c>
       <c r="B180" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C180" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="D180">
         <v>500</v>
@@ -7605,10 +7618,10 @@
         <v>12</v>
       </c>
       <c r="B181" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C181" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="D181">
         <v>500</v>
@@ -7634,10 +7647,10 @@
         <v>12</v>
       </c>
       <c r="B182" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C182" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="D182">
         <v>500</v>
@@ -7666,7 +7679,7 @@
         <v>38</v>
       </c>
       <c r="C183" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="D183">
         <v>500</v>
@@ -7692,10 +7705,10 @@
         <v>12</v>
       </c>
       <c r="B184" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C184" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="D184">
         <v>500</v>
@@ -7724,7 +7737,7 @@
         <v>16</v>
       </c>
       <c r="C185" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D185">
         <v>500</v>
@@ -7753,7 +7766,7 @@
         <v>16</v>
       </c>
       <c r="C186" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D186">
         <v>500</v>
@@ -7782,7 +7795,7 @@
         <v>16</v>
       </c>
       <c r="C187" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D187">
         <v>500</v>
@@ -7808,10 +7821,10 @@
         <v>12</v>
       </c>
       <c r="B188" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C188" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D188">
         <v>500</v>
@@ -7840,7 +7853,7 @@
         <v>28</v>
       </c>
       <c r="C189" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D189">
         <v>500</v>
@@ -7866,10 +7879,10 @@
         <v>12</v>
       </c>
       <c r="B190" t="s">
+        <v>28</v>
+      </c>
+      <c r="C190" t="s">
         <v>42</v>
-      </c>
-      <c r="C190" t="s">
-        <v>16</v>
       </c>
       <c r="D190">
         <v>500</v>
@@ -7898,7 +7911,7 @@
         <v>42</v>
       </c>
       <c r="C191" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D191">
         <v>500</v>
@@ -7927,7 +7940,7 @@
         <v>42</v>
       </c>
       <c r="C192" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="D192">
         <v>500</v>
@@ -7956,7 +7969,7 @@
         <v>42</v>
       </c>
       <c r="C193" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D193">
         <v>500</v>
@@ -7985,7 +7998,7 @@
         <v>42</v>
       </c>
       <c r="C194" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="D194">
         <v>500</v>
@@ -8014,7 +8027,7 @@
         <v>42</v>
       </c>
       <c r="C195" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="D195">
         <v>500</v>
@@ -8043,7 +8056,7 @@
         <v>42</v>
       </c>
       <c r="C196" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D196">
         <v>500</v>
@@ -8072,7 +8085,7 @@
         <v>42</v>
       </c>
       <c r="C197" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="D197">
         <v>500</v>
@@ -8101,7 +8114,7 @@
         <v>42</v>
       </c>
       <c r="C198" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D198">
         <v>500</v>
@@ -8127,10 +8140,10 @@
         <v>12</v>
       </c>
       <c r="B199" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C199" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D199">
         <v>500</v>
@@ -8159,7 +8172,7 @@
         <v>60</v>
       </c>
       <c r="C200" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D200">
         <v>500</v>
@@ -8188,7 +8201,7 @@
         <v>60</v>
       </c>
       <c r="C201" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D201">
         <v>500</v>
@@ -8217,7 +8230,7 @@
         <v>60</v>
       </c>
       <c r="C202" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D202">
         <v>500</v>
@@ -8246,7 +8259,7 @@
         <v>60</v>
       </c>
       <c r="C203" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D203">
         <v>500</v>
@@ -8272,10 +8285,10 @@
         <v>12</v>
       </c>
       <c r="B204" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C204" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D204">
         <v>500</v>
@@ -8304,7 +8317,7 @@
         <v>22</v>
       </c>
       <c r="C205" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D205">
         <v>500</v>
@@ -8333,7 +8346,7 @@
         <v>22</v>
       </c>
       <c r="C206" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D206">
         <v>500</v>
@@ -8359,10 +8372,10 @@
         <v>12</v>
       </c>
       <c r="B207" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="C207" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="D207">
         <v>500</v>
@@ -8391,7 +8404,7 @@
         <v>61</v>
       </c>
       <c r="C208" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D208">
         <v>500</v>
@@ -8420,7 +8433,7 @@
         <v>61</v>
       </c>
       <c r="C209" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D209">
         <v>500</v>
@@ -8446,10 +8459,10 @@
         <v>12</v>
       </c>
       <c r="B210" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C210" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D210">
         <v>500</v>
@@ -8478,7 +8491,7 @@
         <v>64</v>
       </c>
       <c r="C211" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D211">
         <v>500</v>
@@ -8504,10 +8517,10 @@
         <v>12</v>
       </c>
       <c r="B212" t="s">
+        <v>64</v>
+      </c>
+      <c r="C212" t="s">
         <v>24</v>
-      </c>
-      <c r="C212" t="s">
-        <v>64</v>
       </c>
       <c r="D212">
         <v>500</v>
@@ -8536,7 +8549,7 @@
         <v>24</v>
       </c>
       <c r="C213" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D213">
         <v>500</v>
@@ -8562,10 +8575,10 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C214" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="D214">
         <v>500</v>
@@ -8594,7 +8607,7 @@
         <v>18</v>
       </c>
       <c r="C215" t="s">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="D215">
         <v>500</v>
@@ -8623,7 +8636,7 @@
         <v>18</v>
       </c>
       <c r="C216" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="D216">
         <v>500</v>
@@ -8649,10 +8662,10 @@
         <v>12</v>
       </c>
       <c r="B217" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C217" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D217">
         <v>500</v>
@@ -8678,7 +8691,7 @@
         <v>12</v>
       </c>
       <c r="B218" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C218" t="s">
         <v>42</v>
@@ -8707,7 +8720,7 @@
         <v>12</v>
       </c>
       <c r="B219" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C219" t="s">
         <v>42</v>
@@ -8739,7 +8752,7 @@
         <v>62</v>
       </c>
       <c r="C220" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D220">
         <v>500</v>
@@ -8768,7 +8781,7 @@
         <v>62</v>
       </c>
       <c r="C221" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D221">
         <v>500</v>
@@ -8794,10 +8807,10 @@
         <v>12</v>
       </c>
       <c r="B222" t="s">
+        <v>62</v>
+      </c>
+      <c r="C222" t="s">
         <v>65</v>
-      </c>
-      <c r="C222" t="s">
-        <v>60</v>
       </c>
       <c r="D222">
         <v>500</v>
@@ -8826,7 +8839,7 @@
         <v>65</v>
       </c>
       <c r="C223" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D223">
         <v>500</v>
@@ -8855,7 +8868,7 @@
         <v>65</v>
       </c>
       <c r="C224" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D224">
         <v>500</v>
@@ -8884,7 +8897,7 @@
         <v>65</v>
       </c>
       <c r="C225" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D225">
         <v>500</v>
@@ -8910,10 +8923,10 @@
         <v>12</v>
       </c>
       <c r="B226" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C226" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="D226">
         <v>500</v>
@@ -8942,7 +8955,7 @@
         <v>66</v>
       </c>
       <c r="C227" t="s">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="D227">
         <v>500</v>
@@ -8971,7 +8984,7 @@
         <v>66</v>
       </c>
       <c r="C228" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D228">
         <v>500</v>
@@ -9000,7 +9013,7 @@
         <v>66</v>
       </c>
       <c r="C229" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D229">
         <v>500</v>
@@ -9026,10 +9039,10 @@
         <v>12</v>
       </c>
       <c r="B230" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C230" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="D230">
         <v>500</v>
@@ -9058,7 +9071,7 @@
         <v>67</v>
       </c>
       <c r="C231" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D231">
         <v>500</v>
@@ -9084,10 +9097,10 @@
         <v>12</v>
       </c>
       <c r="B232" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C232" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D232">
         <v>500</v>
@@ -9116,7 +9129,7 @@
         <v>68</v>
       </c>
       <c r="C233" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="D233">
         <v>500</v>
@@ -9145,7 +9158,7 @@
         <v>68</v>
       </c>
       <c r="C234" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="D234">
         <v>500</v>
@@ -9174,7 +9187,7 @@
         <v>68</v>
       </c>
       <c r="C235" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="D235">
         <v>500</v>
@@ -9203,7 +9216,7 @@
         <v>68</v>
       </c>
       <c r="C236" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="D236">
         <v>500</v>
@@ -9229,10 +9242,10 @@
         <v>12</v>
       </c>
       <c r="B237" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C237" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="D237">
         <v>500</v>
@@ -9258,10 +9271,10 @@
         <v>12</v>
       </c>
       <c r="B238" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C238" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D238">
         <v>500</v>
@@ -9290,7 +9303,7 @@
         <v>51</v>
       </c>
       <c r="C239" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D239">
         <v>500</v>
@@ -9319,7 +9332,7 @@
         <v>51</v>
       </c>
       <c r="C240" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D240">
         <v>500</v>
@@ -9348,7 +9361,7 @@
         <v>51</v>
       </c>
       <c r="C241" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="D241">
         <v>500</v>
@@ -9374,10 +9387,10 @@
         <v>12</v>
       </c>
       <c r="B242" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="C242" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D242">
         <v>500</v>
@@ -9406,7 +9419,7 @@
         <v>26</v>
       </c>
       <c r="C243" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="D243">
         <v>500</v>
@@ -9432,10 +9445,10 @@
         <v>12</v>
       </c>
       <c r="B244" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="C244" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="D244">
         <v>500</v>
@@ -9464,7 +9477,7 @@
         <v>72</v>
       </c>
       <c r="C245" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="D245">
         <v>500</v>
@@ -9490,10 +9503,10 @@
         <v>12</v>
       </c>
       <c r="B246" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="C246" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D246">
         <v>500</v>
@@ -9522,7 +9535,7 @@
         <v>34</v>
       </c>
       <c r="C247" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D247">
         <v>500</v>
@@ -9548,10 +9561,10 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
+        <v>34</v>
+      </c>
+      <c r="C248" t="s">
         <v>32</v>
-      </c>
-      <c r="C248" t="s">
-        <v>34</v>
       </c>
       <c r="D248">
         <v>500</v>
@@ -9577,10 +9590,10 @@
         <v>12</v>
       </c>
       <c r="B249" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="C249" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D249">
         <v>500</v>
@@ -9609,7 +9622,7 @@
         <v>58</v>
       </c>
       <c r="C250" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D250">
         <v>500</v>
@@ -9638,7 +9651,7 @@
         <v>58</v>
       </c>
       <c r="C251" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D251">
         <v>500</v>
@@ -9667,7 +9680,7 @@
         <v>58</v>
       </c>
       <c r="C252" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="D252">
         <v>500</v>
@@ -9693,7 +9706,7 @@
         <v>12</v>
       </c>
       <c r="B253" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C253" t="s">
         <v>51</v>
@@ -9722,10 +9735,10 @@
         <v>12</v>
       </c>
       <c r="B254" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="C254" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="D254">
         <v>500</v>
@@ -9754,7 +9767,7 @@
         <v>53</v>
       </c>
       <c r="C255" t="s">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="D255">
         <v>500</v>
@@ -9783,7 +9796,7 @@
         <v>53</v>
       </c>
       <c r="C256" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D256">
         <v>500</v>
@@ -9809,10 +9822,10 @@
         <v>12</v>
       </c>
       <c r="B257" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C257" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="D257">
         <v>500</v>
@@ -9838,10 +9851,10 @@
         <v>12</v>
       </c>
       <c r="B258" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="C258" t="s">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="D258">
         <v>500</v>
@@ -9870,7 +9883,7 @@
         <v>36</v>
       </c>
       <c r="C259" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="D259">
         <v>500</v>
@@ -9896,10 +9909,10 @@
         <v>12</v>
       </c>
       <c r="B260" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C260" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D260">
         <v>500</v>
@@ -9928,7 +9941,7 @@
         <v>48</v>
       </c>
       <c r="C261" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D261">
         <v>500</v>
@@ -9957,7 +9970,7 @@
         <v>48</v>
       </c>
       <c r="C262" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D262">
         <v>500</v>
@@ -9986,7 +9999,7 @@
         <v>48</v>
       </c>
       <c r="C263" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D263">
         <v>500</v>
@@ -10012,10 +10025,10 @@
         <v>12</v>
       </c>
       <c r="B264" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C264" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="D264">
         <v>500</v>
@@ -10041,10 +10054,10 @@
         <v>12</v>
       </c>
       <c r="B265" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C265" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D265">
         <v>500</v>
@@ -10070,7 +10083,7 @@
         <v>12</v>
       </c>
       <c r="B266" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C266" t="s">
         <v>22</v>
@@ -10099,10 +10112,10 @@
         <v>12</v>
       </c>
       <c r="B267" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="C267" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D267">
         <v>500</v>
@@ -10131,7 +10144,7 @@
         <v>75</v>
       </c>
       <c r="C268" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D268">
         <v>500</v>
@@ -10157,10 +10170,10 @@
         <v>12</v>
       </c>
       <c r="B269" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C269" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="D269">
         <v>500</v>
@@ -10186,10 +10199,10 @@
         <v>12</v>
       </c>
       <c r="B270" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="C270" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D270">
         <v>500</v>
@@ -10215,10 +10228,10 @@
         <v>12</v>
       </c>
       <c r="B271" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C271" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D271">
         <v>500</v>
@@ -10247,7 +10260,7 @@
         <v>58</v>
       </c>
       <c r="C272" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D272">
         <v>500</v>
@@ -10276,7 +10289,7 @@
         <v>58</v>
       </c>
       <c r="C273" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D273">
         <v>500</v>
@@ -10302,7 +10315,7 @@
         <v>12</v>
       </c>
       <c r="B274" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C274" t="s">
         <v>66</v>
@@ -10331,10 +10344,10 @@
         <v>12</v>
       </c>
       <c r="B275" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C275" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D275">
         <v>500</v>
@@ -10363,7 +10376,7 @@
         <v>68</v>
       </c>
       <c r="C276" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D276">
         <v>500</v>
@@ -10389,10 +10402,10 @@
         <v>12</v>
       </c>
       <c r="B277" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="C277" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D277">
         <v>500</v>
@@ -10418,10 +10431,10 @@
         <v>12</v>
       </c>
       <c r="B278" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="C278" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D278">
         <v>500</v>
@@ -10447,10 +10460,10 @@
         <v>12</v>
       </c>
       <c r="B279" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C279" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="D279">
         <v>500</v>
@@ -10476,7 +10489,7 @@
         <v>12</v>
       </c>
       <c r="B280" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C280" t="s">
         <v>22</v>
@@ -10505,10 +10518,10 @@
         <v>12</v>
       </c>
       <c r="B281" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="C281" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="D281">
         <v>500</v>
@@ -10534,7 +10547,7 @@
         <v>12</v>
       </c>
       <c r="B282" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C282" t="s">
         <v>34</v>
@@ -10563,10 +10576,10 @@
         <v>12</v>
       </c>
       <c r="B283" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="C283" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D283">
         <v>500</v>
@@ -10595,7 +10608,7 @@
         <v>48</v>
       </c>
       <c r="C284" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D284">
         <v>500</v>
@@ -10624,7 +10637,7 @@
         <v>48</v>
       </c>
       <c r="C285" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D285">
         <v>500</v>
@@ -10653,7 +10666,7 @@
         <v>48</v>
       </c>
       <c r="C286" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D286">
         <v>500</v>
@@ -10682,7 +10695,7 @@
         <v>48</v>
       </c>
       <c r="C287" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D287">
         <v>500</v>
@@ -10708,10 +10721,10 @@
         <v>12</v>
       </c>
       <c r="B288" t="s">
+        <v>48</v>
+      </c>
+      <c r="C288" t="s">
         <v>38</v>
-      </c>
-      <c r="C288" t="s">
-        <v>79</v>
       </c>
       <c r="D288">
         <v>500</v>
@@ -10740,7 +10753,7 @@
         <v>38</v>
       </c>
       <c r="C289" t="s">
-        <v>16</v>
+        <v>79</v>
       </c>
       <c r="D289">
         <v>500</v>
@@ -10769,7 +10782,7 @@
         <v>38</v>
       </c>
       <c r="C290" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D290">
         <v>500</v>
@@ -10795,10 +10808,10 @@
         <v>12</v>
       </c>
       <c r="B291" t="s">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="C291" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D291">
         <v>500</v>
@@ -10824,10 +10837,10 @@
         <v>12</v>
       </c>
       <c r="B292" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="C292" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D292">
         <v>500</v>
@@ -10853,10 +10866,10 @@
         <v>12</v>
       </c>
       <c r="B293" t="s">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="C293" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="D293">
         <v>500</v>
@@ -10882,10 +10895,10 @@
         <v>12</v>
       </c>
       <c r="B294" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C294" t="s">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="D294">
         <v>500</v>
@@ -10908,13 +10921,13 @@
     </row>
     <row r="295" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B295" t="s">
         <v>84</v>
       </c>
       <c r="C295" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="D295">
         <v>500</v>
@@ -10940,19 +10953,19 @@
         <v>12</v>
       </c>
       <c r="B296" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C296" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D296">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E296">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="F296">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G296">
         <v>10000000</v>
@@ -10969,19 +10982,19 @@
         <v>12</v>
       </c>
       <c r="B297" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="C297" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D297">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E297">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="F297">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G297">
         <v>10000000</v>
@@ -10998,10 +11011,10 @@
         <v>12</v>
       </c>
       <c r="B298" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C298" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D298">
         <v>10000</v>
@@ -11027,10 +11040,10 @@
         <v>12</v>
       </c>
       <c r="B299" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C299" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="D299">
         <v>10000</v>
@@ -11056,10 +11069,10 @@
         <v>12</v>
       </c>
       <c r="B300" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C300" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D300">
         <v>10000</v>
@@ -11085,10 +11098,10 @@
         <v>12</v>
       </c>
       <c r="B301" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C301" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D301">
         <v>10000</v>
@@ -11114,10 +11127,10 @@
         <v>12</v>
       </c>
       <c r="B302" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C302" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D302">
         <v>10000</v>
@@ -11143,10 +11156,10 @@
         <v>12</v>
       </c>
       <c r="B303" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C303" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D303">
         <v>10000</v>
@@ -11172,10 +11185,10 @@
         <v>12</v>
       </c>
       <c r="B304" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C304" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="D304">
         <v>10000</v>
@@ -11201,10 +11214,10 @@
         <v>12</v>
       </c>
       <c r="B305" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C305" t="s">
-        <v>66</v>
+        <v>18</v>
       </c>
       <c r="D305">
         <v>10000</v>
@@ -11230,10 +11243,10 @@
         <v>12</v>
       </c>
       <c r="B306" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C306" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="D306">
         <v>10000</v>
@@ -11259,10 +11272,10 @@
         <v>12</v>
       </c>
       <c r="B307" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C307" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D307">
         <v>10000</v>
@@ -11288,10 +11301,10 @@
         <v>12</v>
       </c>
       <c r="B308" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C308" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D308">
         <v>10000</v>
@@ -11317,10 +11330,10 @@
         <v>12</v>
       </c>
       <c r="B309" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C309" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D309">
         <v>10000</v>
@@ -11346,10 +11359,10 @@
         <v>12</v>
       </c>
       <c r="B310" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C310" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D310">
         <v>10000</v>
@@ -11375,10 +11388,10 @@
         <v>12</v>
       </c>
       <c r="B311" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C311" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="D311">
         <v>10000</v>
@@ -11396,6 +11409,64 @@
         <v>1000</v>
       </c>
       <c r="I311">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A312" t="s">
+        <v>12</v>
+      </c>
+      <c r="B312" t="s">
+        <v>97</v>
+      </c>
+      <c r="C312" t="s">
+        <v>36</v>
+      </c>
+      <c r="D312">
+        <v>10000</v>
+      </c>
+      <c r="E312">
+        <v>10000</v>
+      </c>
+      <c r="F312">
+        <v>100</v>
+      </c>
+      <c r="G312">
+        <v>10000000</v>
+      </c>
+      <c r="H312">
+        <v>1000</v>
+      </c>
+      <c r="I312">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A313" t="s">
+        <v>12</v>
+      </c>
+      <c r="B313" t="s">
+        <v>98</v>
+      </c>
+      <c r="C313" t="s">
+        <v>34</v>
+      </c>
+      <c r="D313">
+        <v>10000</v>
+      </c>
+      <c r="E313">
+        <v>10000</v>
+      </c>
+      <c r="F313">
+        <v>100</v>
+      </c>
+      <c r="G313">
+        <v>10000000</v>
+      </c>
+      <c r="H313">
+        <v>1000</v>
+      </c>
+      <c r="I313">
         <v>1</v>
       </c>
     </row>
@@ -11407,7 +11478,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68B577B-1347-43AB-A697-F4519763B965}">
-  <dimension ref="A1:G159"/>
+  <dimension ref="A1:C160"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -11938,7 +12009,7 @@
         <v>-661.42899999999997</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>11</v>
       </c>
@@ -11949,7 +12020,7 @@
         <v>-31.263999999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>11</v>
       </c>
@@ -11957,10 +12028,10 @@
         <v>64</v>
       </c>
       <c r="C50">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+        <v>-10.498540930309094</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>11</v>
       </c>
@@ -11968,10 +12039,10 @@
         <v>24</v>
       </c>
       <c r="C51">
-        <v>-50</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+        <v>-20.327868125092017</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>11</v>
       </c>
@@ -11982,7 +12053,7 @@
         <v>-397.63900000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>11</v>
       </c>
@@ -11990,10 +12061,10 @@
         <v>40</v>
       </c>
       <c r="C53">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+        <v>-29.166899245671924</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>11</v>
       </c>
@@ -12003,14 +12074,8 @@
       <c r="C54">
         <v>-211.03200000000001</v>
       </c>
-      <c r="F54" t="s">
-        <v>81</v>
-      </c>
-      <c r="G54">
-        <v>-10.747</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>11</v>
       </c>
@@ -12020,14 +12085,8 @@
       <c r="C55">
         <v>-83.045000000000002</v>
       </c>
-      <c r="F55" t="s">
-        <v>77</v>
-      </c>
-      <c r="G55">
-        <v>-453.32799999999997</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>11</v>
       </c>
@@ -12035,10 +12094,10 @@
         <v>65</v>
       </c>
       <c r="C56">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+        <v>-27.339084185091842</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>11</v>
       </c>
@@ -12049,7 +12108,7 @@
         <v>-99.653999999999982</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>11</v>
       </c>
@@ -12057,10 +12116,10 @@
         <v>67</v>
       </c>
       <c r="C58">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+        <v>-34.696428008002286</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>11</v>
       </c>
@@ -12071,7 +12130,7 @@
         <v>-19.54</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>11</v>
       </c>
@@ -12079,10 +12138,10 @@
         <v>68</v>
       </c>
       <c r="C60">
-        <v>-50</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+        <v>-34.820653312201756</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>11</v>
       </c>
@@ -12093,7 +12152,7 @@
         <v>-55.689</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>11</v>
       </c>
@@ -12104,7 +12163,7 @@
         <v>-110.401</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>11</v>
       </c>
@@ -12112,10 +12171,10 @@
         <v>26</v>
       </c>
       <c r="C63">
-        <v>-20</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+        <v>-13.995883970311864</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>11</v>
       </c>
@@ -12123,7 +12182,7 @@
         <v>72</v>
       </c>
       <c r="C64">
-        <v>-20</v>
+        <v>-9.5558311621502252</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
@@ -12167,7 +12226,7 @@
         <v>71</v>
       </c>
       <c r="C68">
-        <v>-10</v>
+        <v>-12.918429819775348</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
@@ -12274,10 +12333,10 @@
         <v>11</v>
       </c>
       <c r="B78" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C78">
-        <v>0</v>
+        <v>-10.747</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
@@ -12934,7 +12993,7 @@
         <v>12</v>
       </c>
       <c r="B138" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -12978,7 +13037,7 @@
         <v>12</v>
       </c>
       <c r="B142" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -12989,7 +13048,7 @@
         <v>12</v>
       </c>
       <c r="B143" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C143">
         <v>0</v>
@@ -13000,7 +13059,7 @@
         <v>12</v>
       </c>
       <c r="B144" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C144">
         <v>0</v>
@@ -13011,7 +13070,7 @@
         <v>12</v>
       </c>
       <c r="B145" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C145">
         <v>0</v>
@@ -13022,7 +13081,7 @@
         <v>12</v>
       </c>
       <c r="B146" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C146">
         <v>0</v>
@@ -13033,7 +13092,7 @@
         <v>12</v>
       </c>
       <c r="B147" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C147">
         <v>0</v>
@@ -13044,7 +13103,7 @@
         <v>12</v>
       </c>
       <c r="B148" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C148">
         <v>0</v>
@@ -13055,7 +13114,7 @@
         <v>12</v>
       </c>
       <c r="B149" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -13066,7 +13125,7 @@
         <v>12</v>
       </c>
       <c r="B150" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C150">
         <v>0</v>
@@ -13077,7 +13136,7 @@
         <v>12</v>
       </c>
       <c r="B151" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C151">
         <v>0</v>
@@ -13088,7 +13147,7 @@
         <v>12</v>
       </c>
       <c r="B152" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C152">
         <v>0</v>
@@ -13099,7 +13158,7 @@
         <v>12</v>
       </c>
       <c r="B153" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C153">
         <v>0</v>
@@ -13110,7 +13169,7 @@
         <v>12</v>
       </c>
       <c r="B154" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C154">
         <v>0</v>
@@ -13121,7 +13180,7 @@
         <v>12</v>
       </c>
       <c r="B155" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C155">
         <v>0</v>
@@ -13132,7 +13191,7 @@
         <v>12</v>
       </c>
       <c r="B156" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -13143,7 +13202,7 @@
         <v>12</v>
       </c>
       <c r="B157" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C157">
         <v>0</v>
@@ -13151,10 +13210,10 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B158" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -13162,12 +13221,23 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B159" t="s">
         <v>84</v>
       </c>
       <c r="C159">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A160" t="s">
+        <v>12</v>
+      </c>
+      <c r="B160" t="s">
+        <v>84</v>
+      </c>
+      <c r="C160">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add import route over BY
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640808F7-3D5D-4B0C-932E-02E9AB3AEDB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A51C345F-A8A2-4127-9B75-711C89601CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1673" uniqueCount="99">
   <si>
     <t>Commodities</t>
   </si>
@@ -694,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B0CB446-BDDD-415D-AF22-2CEB1FE45CA5}">
-  <dimension ref="A1:A79"/>
+  <dimension ref="A1:A81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -1090,6 +1090,16 @@
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1124,7 +1134,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B157"/>
+  <dimension ref="A1:B158"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2381,6 +2391,14 @@
       </c>
       <c r="B157" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>53</v>
+      </c>
+      <c r="B158" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -2390,7 +2408,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I313"/>
+  <dimension ref="A1:I314"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -6110,16 +6128,16 @@
         <v>11</v>
       </c>
       <c r="B129" t="s">
+        <v>53</v>
+      </c>
+      <c r="C129" t="s">
         <v>75</v>
       </c>
-      <c r="C129" t="s">
-        <v>26</v>
-      </c>
       <c r="D129">
-        <v>118.77099999999999</v>
+        <v>439.27749999999992</v>
       </c>
       <c r="E129">
-        <v>118.77099999999999</v>
+        <v>439.27749999999992</v>
       </c>
       <c r="F129">
         <v>1</v>
@@ -6139,16 +6157,16 @@
         <v>11</v>
       </c>
       <c r="B130" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C130" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="D130">
-        <v>486.91</v>
+        <v>118.77099999999999</v>
       </c>
       <c r="E130">
-        <v>486.91</v>
+        <v>118.77099999999999</v>
       </c>
       <c r="F130">
         <v>1</v>
@@ -6168,16 +6186,16 @@
         <v>11</v>
       </c>
       <c r="B131" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="C131" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D131">
-        <v>144.17500000000001</v>
+        <v>486.91</v>
       </c>
       <c r="E131">
-        <v>144.17500000000001</v>
+        <v>486.91</v>
       </c>
       <c r="F131">
         <v>1</v>
@@ -6197,16 +6215,16 @@
         <v>11</v>
       </c>
       <c r="B132" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C132" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D132">
-        <v>49.494</v>
+        <v>144.17500000000001</v>
       </c>
       <c r="E132">
-        <v>49.494</v>
+        <v>144.17500000000001</v>
       </c>
       <c r="F132">
         <v>1</v>
@@ -6229,13 +6247,13 @@
         <v>58</v>
       </c>
       <c r="C133" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D133">
-        <v>816.06700000000012</v>
+        <v>49.494</v>
       </c>
       <c r="E133">
-        <v>816.06700000000012</v>
+        <v>49.494</v>
       </c>
       <c r="F133">
         <v>1</v>
@@ -6258,13 +6276,13 @@
         <v>58</v>
       </c>
       <c r="C134" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D134">
-        <v>188.88749999999999</v>
+        <v>816.06700000000012</v>
       </c>
       <c r="E134">
-        <v>188.88749999999999</v>
+        <v>816.06700000000012</v>
       </c>
       <c r="F134">
         <v>1</v>
@@ -6284,16 +6302,16 @@
         <v>11</v>
       </c>
       <c r="B135" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C135" t="s">
         <v>66</v>
       </c>
       <c r="D135">
-        <v>89.716999999999999</v>
+        <v>188.88749999999999</v>
       </c>
       <c r="E135">
-        <v>89.716999999999999</v>
+        <v>188.88749999999999</v>
       </c>
       <c r="F135">
         <v>1</v>
@@ -6313,16 +6331,16 @@
         <v>11</v>
       </c>
       <c r="B136" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C136" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D136">
-        <v>170.63749999999999</v>
+        <v>89.716999999999999</v>
       </c>
       <c r="E136">
-        <v>170.63749999999999</v>
+        <v>89.716999999999999</v>
       </c>
       <c r="F136">
         <v>1</v>
@@ -6345,13 +6363,13 @@
         <v>68</v>
       </c>
       <c r="C137" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D137">
-        <v>12.1837</v>
+        <v>170.63749999999999</v>
       </c>
       <c r="E137">
-        <v>12.1837</v>
+        <v>170.63749999999999</v>
       </c>
       <c r="F137">
         <v>1</v>
@@ -6371,16 +6389,16 @@
         <v>11</v>
       </c>
       <c r="B138" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="C138" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D138">
-        <v>256.15699999999998</v>
+        <v>12.1837</v>
       </c>
       <c r="E138">
-        <v>256.15699999999998</v>
+        <v>12.1837</v>
       </c>
       <c r="F138">
         <v>1</v>
@@ -6400,16 +6418,16 @@
         <v>11</v>
       </c>
       <c r="B139" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="C139" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D139">
-        <v>61.32</v>
+        <v>256.15699999999998</v>
       </c>
       <c r="E139">
-        <v>61.32</v>
+        <v>256.15699999999998</v>
       </c>
       <c r="F139">
         <v>1</v>
@@ -10460,10 +10478,10 @@
         <v>12</v>
       </c>
       <c r="B279" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C279" t="s">
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="D279">
         <v>500</v>
@@ -10489,7 +10507,7 @@
         <v>12</v>
       </c>
       <c r="B280" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C280" t="s">
         <v>22</v>
@@ -10518,10 +10536,10 @@
         <v>12</v>
       </c>
       <c r="B281" t="s">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="C281" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D281">
         <v>500</v>
@@ -10547,7 +10565,7 @@
         <v>12</v>
       </c>
       <c r="B282" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C282" t="s">
         <v>34</v>
@@ -10576,10 +10594,10 @@
         <v>12</v>
       </c>
       <c r="B283" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C283" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D283">
         <v>500</v>
@@ -10608,7 +10626,7 @@
         <v>48</v>
       </c>
       <c r="C284" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D284">
         <v>500</v>
@@ -10637,7 +10655,7 @@
         <v>48</v>
       </c>
       <c r="C285" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D285">
         <v>500</v>
@@ -10666,7 +10684,7 @@
         <v>48</v>
       </c>
       <c r="C286" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D286">
         <v>500</v>
@@ -10695,7 +10713,7 @@
         <v>48</v>
       </c>
       <c r="C287" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D287">
         <v>500</v>
@@ -10721,10 +10739,10 @@
         <v>12</v>
       </c>
       <c r="B288" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C288" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="D288">
         <v>500</v>
@@ -10753,7 +10771,7 @@
         <v>38</v>
       </c>
       <c r="C289" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="D289">
         <v>500</v>
@@ -10782,7 +10800,7 @@
         <v>38</v>
       </c>
       <c r="C290" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D290">
         <v>500</v>
@@ -10808,10 +10826,10 @@
         <v>12</v>
       </c>
       <c r="B291" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="C291" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D291">
         <v>500</v>
@@ -10837,10 +10855,10 @@
         <v>12</v>
       </c>
       <c r="B292" t="s">
+        <v>20</v>
+      </c>
+      <c r="C292" t="s">
         <v>74</v>
-      </c>
-      <c r="C292" t="s">
-        <v>22</v>
       </c>
       <c r="D292">
         <v>500</v>
@@ -10866,10 +10884,10 @@
         <v>12</v>
       </c>
       <c r="B293" t="s">
+        <v>77</v>
+      </c>
+      <c r="C293" t="s">
         <v>20</v>
-      </c>
-      <c r="C293" t="s">
-        <v>74</v>
       </c>
       <c r="D293">
         <v>500</v>
@@ -10895,10 +10913,10 @@
         <v>12</v>
       </c>
       <c r="B294" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C294" t="s">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="D294">
         <v>500</v>
@@ -10927,7 +10945,7 @@
         <v>84</v>
       </c>
       <c r="C295" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="D295">
         <v>500</v>
@@ -10953,10 +10971,10 @@
         <v>12</v>
       </c>
       <c r="B296" t="s">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="C296" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="D296">
         <v>500</v>
@@ -10982,19 +11000,19 @@
         <v>12</v>
       </c>
       <c r="B297" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="C297" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="D297">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="E297">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="F297">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G297">
         <v>10000000</v>
@@ -11011,10 +11029,10 @@
         <v>12</v>
       </c>
       <c r="B298" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C298" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D298">
         <v>10000</v>
@@ -11040,10 +11058,10 @@
         <v>12</v>
       </c>
       <c r="B299" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C299" t="s">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="D299">
         <v>10000</v>
@@ -11069,10 +11087,10 @@
         <v>12</v>
       </c>
       <c r="B300" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C300" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="D300">
         <v>10000</v>
@@ -11098,10 +11116,10 @@
         <v>12</v>
       </c>
       <c r="B301" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C301" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="D301">
         <v>10000</v>
@@ -11127,10 +11145,10 @@
         <v>12</v>
       </c>
       <c r="B302" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C302" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="D302">
         <v>10000</v>
@@ -11156,10 +11174,10 @@
         <v>12</v>
       </c>
       <c r="B303" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C303" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="D303">
         <v>10000</v>
@@ -11185,10 +11203,10 @@
         <v>12</v>
       </c>
       <c r="B304" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C304" t="s">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="D304">
         <v>10000</v>
@@ -11214,10 +11232,10 @@
         <v>12</v>
       </c>
       <c r="B305" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C305" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D305">
         <v>10000</v>
@@ -11243,10 +11261,10 @@
         <v>12</v>
       </c>
       <c r="B306" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C306" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="D306">
         <v>10000</v>
@@ -11272,10 +11290,10 @@
         <v>12</v>
       </c>
       <c r="B307" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C307" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D307">
         <v>10000</v>
@@ -11301,10 +11319,10 @@
         <v>12</v>
       </c>
       <c r="B308" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C308" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D308">
         <v>10000</v>
@@ -11330,10 +11348,10 @@
         <v>12</v>
       </c>
       <c r="B309" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C309" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D309">
         <v>10000</v>
@@ -11359,10 +11377,10 @@
         <v>12</v>
       </c>
       <c r="B310" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C310" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D310">
         <v>10000</v>
@@ -11388,10 +11406,10 @@
         <v>12</v>
       </c>
       <c r="B311" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C311" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="D311">
         <v>10000</v>
@@ -11417,10 +11435,10 @@
         <v>12</v>
       </c>
       <c r="B312" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C312" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D312">
         <v>10000</v>
@@ -11446,19 +11464,19 @@
         <v>12</v>
       </c>
       <c r="B313" t="s">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="C313" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D313">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E313">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="F313">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G313">
         <v>10000000</v>
@@ -11467,6 +11485,35 @@
         <v>1000</v>
       </c>
       <c r="I313">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A314" t="s">
+        <v>12</v>
+      </c>
+      <c r="B314" t="s">
+        <v>75</v>
+      </c>
+      <c r="C314" t="s">
+        <v>30</v>
+      </c>
+      <c r="D314">
+        <v>500</v>
+      </c>
+      <c r="E314">
+        <v>500</v>
+      </c>
+      <c r="F314">
+        <v>1</v>
+      </c>
+      <c r="G314">
+        <v>10000000</v>
+      </c>
+      <c r="H314">
+        <v>1000</v>
+      </c>
+      <c r="I314">
         <v>1</v>
       </c>
     </row>
@@ -11478,7 +11525,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68B577B-1347-43AB-A697-F4519763B965}">
-  <dimension ref="A1:C160"/>
+  <dimension ref="A1:C162"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -13007,7 +13054,7 @@
         <v>69</v>
       </c>
       <c r="C139">
-        <v>0</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.35">
@@ -13238,6 +13285,28 @@
         <v>84</v>
       </c>
       <c r="C160">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A161" t="s">
+        <v>11</v>
+      </c>
+      <c r="B161" t="s">
+        <v>75</v>
+      </c>
+      <c r="C161">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>12</v>
+      </c>
+      <c r="B162" t="s">
+        <v>75</v>
+      </c>
+      <c r="C162">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
test different commodity shortage cost
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC30B68-F149-49D2-9BD4-63DBDE1D0480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76DD410E-E2B9-4E73-A272-4C5B0151C4A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
transfer from network to excess not working
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update_methane_LNG_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76DD410E-E2B9-4E73-A272-4C5B0151C4A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06798385-13A4-421A-96D7-F1160EEE40FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -11156,7 +11156,7 @@
         <v>10000</v>
       </c>
       <c r="F303">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G303">
         <v>10000000</v>
@@ -11185,7 +11185,7 @@
         <v>10000</v>
       </c>
       <c r="F304">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G304">
         <v>10000000</v>

</xml_diff>